<commit_message>
coaching: pull 09-12.07, Maciek 5K PB 19:49 + recalib plan W13-20, Teneryfa camp, Sheets push
- Tomasz 09-12.07: long 21.4, easy 9.35, signature 2x5km @4:05/3:58 (2. hard T9)
- Maciek 5K TEST 19:49 (VDOT 52-53, -1:25 vs 21:14), negative split analiza
- Plan Maciek recalib W13-W20 do Praskiego (xlsx tab Plan, akcenty pod VDOT 52-53)
- Teneryfa obóz 10-24.08: 2 longi wysokościowe (13+18.08) Tomasz T14/T15 + Maciek W17/W18
- scripts/push_maciek_sheet.py: mirror xlsx -> Google Sheet (SA), skill maciek-update

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/maciek_plan_full.xlsx
+++ b/data/maciek_plan_full.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,8 +121,57 @@
       <color rgb="008A6D00"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F2A37"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="005C5C5C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C77700"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C62828"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001565C0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00333333"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00BF5B00"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00AD1457"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -189,6 +238,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE7EF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -230,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -343,6 +397,23 @@
     <xf numFmtId="49" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -708,7 +779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H156"/>
+  <dimension ref="A1:H230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4430,668 +4501,2940 @@
       <c r="H126" s="6" t="inlineStr"/>
     </row>
     <row r="127">
-      <c r="A127" s="33" t="inlineStr">
-        <is>
-          <t>★ DALEJ = SZKIC. Po teście 5K (12.07) recalibrujemy tempa i dopisujemy szczegóły kolejnego bloku.</t>
-        </is>
-      </c>
-      <c r="B127" s="33" t="inlineStr"/>
-      <c r="C127" s="34" t="inlineStr"/>
-      <c r="D127" s="33" t="inlineStr"/>
-      <c r="E127" s="33" t="inlineStr"/>
-      <c r="F127" s="33" t="inlineStr"/>
-      <c r="G127" s="33" t="inlineStr"/>
-      <c r="H127" s="34" t="inlineStr"/>
+      <c r="A127" s="38" t="inlineStr">
+        <is>
+          <t>TYDZIEŃ 13 — HM-SPEC ENTRY (recalib VDOT 52-53, ~88 km) · po 5K TT 19:49</t>
+        </is>
+      </c>
+      <c r="B127" s="39" t="n"/>
+      <c r="C127" s="39" t="n"/>
+      <c r="D127" s="39" t="n"/>
+      <c r="E127" s="39" t="n"/>
+      <c r="F127" s="39" t="n"/>
+      <c r="G127" s="39" t="n"/>
+      <c r="H127" s="39" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="28" t="inlineStr">
-        <is>
-          <t>■ BLOK 2: HM-SPECIFIC (13.07-9.08) — dłuższe progi + HM-pace longi (szkic)</t>
-        </is>
-      </c>
-      <c r="B128" s="28" t="inlineStr"/>
-      <c r="C128" s="29" t="inlineStr"/>
-      <c r="D128" s="28" t="inlineStr"/>
-      <c r="E128" s="28" t="inlineStr"/>
-      <c r="F128" s="28" t="inlineStr"/>
-      <c r="G128" s="28" t="inlineStr"/>
-      <c r="H128" s="29" t="inlineStr"/>
+      <c r="A128" s="40" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B128" s="40" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="C128" s="40" t="inlineStr">
+        <is>
+          <t>Trening</t>
+        </is>
+      </c>
+      <c r="D128" s="40" t="inlineStr">
+        <is>
+          <t>Tempo /km</t>
+        </is>
+      </c>
+      <c r="E128" s="40" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="F128" s="40" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G128" s="40" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="H128" s="40" t="inlineStr">
+        <is>
+          <t>Notatki / feedback</t>
+        </is>
+      </c>
     </row>
     <row r="129">
-      <c r="A129" s="9" t="inlineStr">
+      <c r="A129" s="41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B129" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C129" s="41" t="inlineStr">
+        <is>
+          <t>Recovery 10 km (po 5K TT z nd)</t>
+        </is>
+      </c>
+      <c r="D129" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E129" s="41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F129" s="41" t="inlineStr"/>
+      <c r="G129" s="41" t="inlineStr">
+        <is>
+          <t>13.07</t>
+        </is>
+      </c>
+      <c r="H129" s="41" t="inlineStr">
+        <is>
+          <t>luźno, nogi po teście</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="41" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B130" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C130" s="41" t="inlineStr">
+        <is>
+          <t>Easy 12 km + 6×100 m stride</t>
+        </is>
+      </c>
+      <c r="D130" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E130" s="41" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F130" s="41" t="inlineStr"/>
+      <c r="G130" s="41" t="inlineStr">
+        <is>
+          <t>14.07</t>
+        </is>
+      </c>
+      <c r="H130" s="41" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="43" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B131" s="44" t="inlineStr">
+        <is>
+          <t>THRESHOLD</t>
+        </is>
+      </c>
+      <c r="C131" s="43" t="inlineStr">
+        <is>
+          <t>2 WU → 2×4 km @ 4:08–4:12 (800 jog) → 2 CD</t>
+        </is>
+      </c>
+      <c r="D131" s="43" t="inlineStr">
+        <is>
+          <t>4:08–4:12</t>
+        </is>
+      </c>
+      <c r="E131" s="43" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F131" s="43" t="inlineStr"/>
+      <c r="G131" s="43" t="inlineStr">
+        <is>
+          <t>15.07</t>
+        </is>
+      </c>
+      <c r="H131" s="43" t="inlineStr">
+        <is>
+          <t>NA TEMPIE od 1. odcinka</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B132" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C132" s="41" t="inlineStr">
+        <is>
+          <t>Easy 10 km</t>
+        </is>
+      </c>
+      <c r="D132" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E132" s="41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F132" s="41" t="inlineStr"/>
+      <c r="G132" s="41" t="inlineStr">
+        <is>
+          <t>16.07</t>
+        </is>
+      </c>
+      <c r="H132" s="41" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="45" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B133" s="46" t="inlineStr">
+        <is>
+          <t>VO2max</t>
+        </is>
+      </c>
+      <c r="C133" s="45" t="inlineStr">
+        <is>
+          <t>3 WU → 5×1000 @ 3:50 (400 jog) → 2 CD</t>
+        </is>
+      </c>
+      <c r="D133" s="45" t="inlineStr">
+        <is>
+          <t>3:48–3:53</t>
+        </is>
+      </c>
+      <c r="E133" s="45" t="inlineStr">
+        <is>
+          <t>12,5</t>
+        </is>
+      </c>
+      <c r="F133" s="45" t="inlineStr"/>
+      <c r="G133" s="45" t="inlineStr">
+        <is>
+          <t>18.07</t>
+        </is>
+      </c>
+      <c r="H133" s="45" t="inlineStr">
+        <is>
+          <t>pas piersiowy na HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B134" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C134" s="41" t="inlineStr">
+        <is>
+          <t>Recovery 8 km</t>
+        </is>
+      </c>
+      <c r="D134" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E134" s="41" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F134" s="41" t="inlineStr"/>
+      <c r="G134" s="41" t="inlineStr">
+        <is>
+          <t>19.07</t>
+        </is>
+      </c>
+      <c r="H134" s="41" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="47" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B135" s="48" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="C135" s="47" t="inlineStr">
+        <is>
+          <t>24 km, ostatnie 6 km @ HM-pace 4:12</t>
+        </is>
+      </c>
+      <c r="D135" s="47" t="inlineStr">
+        <is>
+          <t>5:40–6:15 → 4:12</t>
+        </is>
+      </c>
+      <c r="E135" s="47" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F135" s="47" t="inlineStr"/>
+      <c r="G135" s="47" t="inlineStr">
+        <is>
+          <t>20.07</t>
+        </is>
+      </c>
+      <c r="H135" s="47" t="inlineStr">
+        <is>
+          <t>long spływa na pon</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="49" t="n"/>
+      <c r="B136" s="49" t="n"/>
+      <c r="C136" s="49" t="n"/>
+      <c r="D136" s="50" t="inlineStr">
+        <is>
+          <t>SUMA km:</t>
+        </is>
+      </c>
+      <c r="E136" s="50" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="F136" s="49" t="n"/>
+      <c r="G136" s="49" t="n"/>
+      <c r="H136" s="50" t="inlineStr">
+        <is>
+          <t>2 jakości + long z finishem HM. Easy MUSI być easy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="38" t="inlineStr">
+        <is>
+          <t>TYDZIEŃ 14 — NAJWIĘKSZY BLOK HM-SPEC (~88 km)</t>
+        </is>
+      </c>
+      <c r="B137" s="39" t="n"/>
+      <c r="C137" s="39" t="n"/>
+      <c r="D137" s="39" t="n"/>
+      <c r="E137" s="39" t="n"/>
+      <c r="F137" s="39" t="n"/>
+      <c r="G137" s="39" t="n"/>
+      <c r="H137" s="39" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="40" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B138" s="40" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="C138" s="40" t="inlineStr">
+        <is>
+          <t>Trening</t>
+        </is>
+      </c>
+      <c r="D138" s="40" t="inlineStr">
+        <is>
+          <t>Tempo /km</t>
+        </is>
+      </c>
+      <c r="E138" s="40" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="F138" s="40" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G138" s="40" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="H138" s="40" t="inlineStr">
+        <is>
+          <t>Notatki / feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B139" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C139" s="41" t="inlineStr">
+        <is>
+          <t>Easy 12 km + strides</t>
+        </is>
+      </c>
+      <c r="D139" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E139" s="41" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F139" s="41" t="inlineStr"/>
+      <c r="G139" s="41" t="inlineStr">
+        <is>
+          <t>20.07</t>
+        </is>
+      </c>
+      <c r="H139" s="41" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B140" s="44" t="inlineStr">
+        <is>
+          <t>THRESHOLD</t>
+        </is>
+      </c>
+      <c r="C140" s="43" t="inlineStr">
+        <is>
+          <t>PRÓG CIĄGŁY 6 km @ 4:12 (WU 3 + CD 3)</t>
+        </is>
+      </c>
+      <c r="D140" s="43" t="inlineStr">
+        <is>
+          <t>4:10–4:12</t>
+        </is>
+      </c>
+      <c r="E140" s="43" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F140" s="43" t="inlineStr"/>
+      <c r="G140" s="43" t="inlineStr">
+        <is>
+          <t>21.07</t>
+        </is>
+      </c>
+      <c r="H140" s="43" t="inlineStr">
+        <is>
+          <t>trening trzymania tempa</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B141" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C141" s="41" t="inlineStr">
+        <is>
+          <t>Easy 10 km</t>
+        </is>
+      </c>
+      <c r="D141" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E141" s="41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F141" s="41" t="inlineStr"/>
+      <c r="G141" s="41" t="inlineStr">
+        <is>
+          <t>22.07</t>
+        </is>
+      </c>
+      <c r="H141" s="41" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="51" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B142" s="52" t="inlineStr">
+        <is>
+          <t>TOUGHNESS</t>
+        </is>
+      </c>
+      <c r="C142" s="51" t="inlineStr">
+        <is>
+          <t>6×1000 @ 3:48–3:52, rec 200 m KRÓTKA (WU3+CD2)</t>
+        </is>
+      </c>
+      <c r="D142" s="51" t="inlineStr">
+        <is>
+          <t>3:48–3:52</t>
+        </is>
+      </c>
+      <c r="E142" s="51" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F142" s="51" t="inlineStr"/>
+      <c r="G142" s="51" t="inlineStr">
+        <is>
+          <t>23.07</t>
+        </is>
+      </c>
+      <c r="H142" s="51" t="inlineStr">
+        <is>
+          <t>limiter — tolerancja wys. HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="41" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B143" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C143" s="41" t="inlineStr">
+        <is>
+          <t>Easy 8 km</t>
+        </is>
+      </c>
+      <c r="D143" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E143" s="41" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F143" s="41" t="inlineStr"/>
+      <c r="G143" s="41" t="inlineStr">
+        <is>
+          <t>24.07</t>
+        </is>
+      </c>
+      <c r="H143" s="41" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="51" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B144" s="52" t="inlineStr">
+        <is>
+          <t>HILL</t>
+        </is>
+      </c>
+      <c r="C144" s="51" t="inlineStr">
+        <is>
+          <t>Easy 6 + 8× podbieg 40 s + 2 CD</t>
+        </is>
+      </c>
+      <c r="D144" s="51" t="inlineStr">
+        <is>
+          <t>wysiłek</t>
+        </is>
+      </c>
+      <c r="E144" s="51" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F144" s="51" t="inlineStr"/>
+      <c r="G144" s="51" t="inlineStr">
+        <is>
+          <t>25.07</t>
+        </is>
+      </c>
+      <c r="H144" s="51" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="47" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B145" s="48" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="C145" s="47" t="inlineStr">
+        <is>
+          <t>26 km z 10 km @ HM-pace 4:12</t>
+        </is>
+      </c>
+      <c r="D145" s="47" t="inlineStr">
+        <is>
+          <t>5:40–6:15 → 4:12</t>
+        </is>
+      </c>
+      <c r="E145" s="47" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="F145" s="47" t="inlineStr"/>
+      <c r="G145" s="47" t="inlineStr">
+        <is>
+          <t>26.07</t>
+        </is>
+      </c>
+      <c r="H145" s="47" t="inlineStr">
+        <is>
+          <t>cap longa 26–28</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="49" t="n"/>
+      <c r="B146" s="49" t="n"/>
+      <c r="C146" s="49" t="n"/>
+      <c r="D146" s="50" t="inlineStr">
+        <is>
+          <t>SUMA km:</t>
+        </is>
+      </c>
+      <c r="E146" s="50" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="F146" s="49" t="n"/>
+      <c r="G146" s="49" t="n"/>
+      <c r="H146" s="50" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="38" t="inlineStr">
+        <is>
+          <t>TYDZIEŃ 15 — HM-SPEC (dłuższe bloki race-pace, ~86 km)</t>
+        </is>
+      </c>
+      <c r="B147" s="39" t="n"/>
+      <c r="C147" s="39" t="n"/>
+      <c r="D147" s="39" t="n"/>
+      <c r="E147" s="39" t="n"/>
+      <c r="F147" s="39" t="n"/>
+      <c r="G147" s="39" t="n"/>
+      <c r="H147" s="39" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="40" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B148" s="40" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="C148" s="40" t="inlineStr">
+        <is>
+          <t>Trening</t>
+        </is>
+      </c>
+      <c r="D148" s="40" t="inlineStr">
+        <is>
+          <t>Tempo /km</t>
+        </is>
+      </c>
+      <c r="E148" s="40" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="F148" s="40" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G148" s="40" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="H148" s="40" t="inlineStr">
+        <is>
+          <t>Notatki / feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B149" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C149" s="41" t="inlineStr">
+        <is>
+          <t>Easy 12 km + strides</t>
+        </is>
+      </c>
+      <c r="D149" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E149" s="41" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F149" s="41" t="inlineStr"/>
+      <c r="G149" s="41" t="inlineStr">
+        <is>
+          <t>27.07</t>
+        </is>
+      </c>
+      <c r="H149" s="41" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B150" s="44" t="inlineStr">
+        <is>
+          <t>THRESHOLD</t>
+        </is>
+      </c>
+      <c r="C150" s="43" t="inlineStr">
+        <is>
+          <t>2 WU → 2×5 km @ 4:10 (800 jog) → 2 CD</t>
+        </is>
+      </c>
+      <c r="D150" s="43" t="inlineStr">
+        <is>
+          <t>4:08–4:12</t>
+        </is>
+      </c>
+      <c r="E150" s="43" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F150" s="43" t="inlineStr"/>
+      <c r="G150" s="43" t="inlineStr">
+        <is>
+          <t>28.07</t>
+        </is>
+      </c>
+      <c r="H150" s="43" t="inlineStr">
+        <is>
+          <t>tempo od startu odcinka</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B151" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C151" s="41" t="inlineStr">
+        <is>
+          <t>Easy 12 km</t>
+        </is>
+      </c>
+      <c r="D151" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E151" s="41" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F151" s="41" t="inlineStr"/>
+      <c r="G151" s="41" t="inlineStr">
+        <is>
+          <t>29.07</t>
+        </is>
+      </c>
+      <c r="H151" s="41" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="45" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B152" s="46" t="inlineStr">
+        <is>
+          <t>VO2max</t>
+        </is>
+      </c>
+      <c r="C152" s="45" t="inlineStr">
+        <is>
+          <t>3 WU → 8×800 @ 3:04 (400 jog) → 2 CD</t>
+        </is>
+      </c>
+      <c r="D152" s="45" t="inlineStr">
+        <is>
+          <t>3:02–3:06</t>
+        </is>
+      </c>
+      <c r="E152" s="45" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F152" s="45" t="inlineStr"/>
+      <c r="G152" s="45" t="inlineStr">
+        <is>
+          <t>30.07</t>
+        </is>
+      </c>
+      <c r="H152" s="45" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="41" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B153" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C153" s="41" t="inlineStr">
+        <is>
+          <t>Easy 8 km</t>
+        </is>
+      </c>
+      <c r="D153" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E153" s="41" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F153" s="41" t="inlineStr"/>
+      <c r="G153" s="41" t="inlineStr">
+        <is>
+          <t>31.07</t>
+        </is>
+      </c>
+      <c r="H153" s="41" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B154" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C154" s="41" t="inlineStr">
+        <is>
+          <t>REST lub easy 6 km</t>
+        </is>
+      </c>
+      <c r="D154" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E154" s="41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F154" s="41" t="inlineStr"/>
+      <c r="G154" s="41" t="inlineStr">
+        <is>
+          <t>1.08</t>
+        </is>
+      </c>
+      <c r="H154" s="41" t="inlineStr">
+        <is>
+          <t>sobota luz</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="47" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B155" s="48" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="C155" s="47" t="inlineStr">
+        <is>
+          <t>24 km z 12 km @ HM-pace 4:12</t>
+        </is>
+      </c>
+      <c r="D155" s="47" t="inlineStr">
+        <is>
+          <t>5:40–6:15 → 4:12</t>
+        </is>
+      </c>
+      <c r="E155" s="47" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F155" s="47" t="inlineStr"/>
+      <c r="G155" s="47" t="inlineStr">
+        <is>
+          <t>2.08</t>
+        </is>
+      </c>
+      <c r="H155" s="47" t="inlineStr">
+        <is>
+          <t>najdłuższy blok race-pace</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="49" t="n"/>
+      <c r="B156" s="49" t="n"/>
+      <c r="C156" s="49" t="n"/>
+      <c r="D156" s="50" t="inlineStr">
+        <is>
+          <t>SUMA km:</t>
+        </is>
+      </c>
+      <c r="E156" s="50" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="F156" s="49" t="n"/>
+      <c r="G156" s="49" t="n"/>
+      <c r="H156" s="50" t="inlineStr">
+        <is>
+          <t>Po tym tyg — deload + 3K TT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="38" t="inlineStr">
+        <is>
+          <t>TYDZIEŃ 16 — DELOAD + 3K TT CHECK (recalibracja, ~66 km)</t>
+        </is>
+      </c>
+      <c r="B157" s="39" t="n"/>
+      <c r="C157" s="39" t="n"/>
+      <c r="D157" s="39" t="n"/>
+      <c r="E157" s="39" t="n"/>
+      <c r="F157" s="39" t="n"/>
+      <c r="G157" s="39" t="n"/>
+      <c r="H157" s="39" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="40" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B158" s="40" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="C158" s="40" t="inlineStr">
+        <is>
+          <t>Trening</t>
+        </is>
+      </c>
+      <c r="D158" s="40" t="inlineStr">
+        <is>
+          <t>Tempo /km</t>
+        </is>
+      </c>
+      <c r="E158" s="40" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="F158" s="40" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G158" s="40" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="H158" s="40" t="inlineStr">
+        <is>
+          <t>Notatki / feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B159" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C159" s="41" t="inlineStr">
+        <is>
+          <t>Easy 12 km</t>
+        </is>
+      </c>
+      <c r="D159" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E159" s="41" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F159" s="41" t="inlineStr"/>
+      <c r="G159" s="41" t="inlineStr">
+        <is>
+          <t>3.08</t>
+        </is>
+      </c>
+      <c r="H159" s="41" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="41" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B160" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C160" s="41" t="inlineStr">
+        <is>
+          <t>Easy 8 km + 4×100 stride</t>
+        </is>
+      </c>
+      <c r="D160" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E160" s="41" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F160" s="41" t="inlineStr"/>
+      <c r="G160" s="41" t="inlineStr">
+        <is>
+          <t>4.08</t>
+        </is>
+      </c>
+      <c r="H160" s="41" t="inlineStr">
+        <is>
+          <t>primer przed TT</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="45" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B161" s="46" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="C161" s="45" t="inlineStr">
+        <is>
+          <t>3K TT — RÓWNYM TEMPEM, wyjść 3:55! (WU 3 + CD 3)</t>
+        </is>
+      </c>
+      <c r="D161" s="45" t="inlineStr">
+        <is>
+          <t>3:52–3:55</t>
+        </is>
+      </c>
+      <c r="E161" s="45" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F161" s="45" t="inlineStr"/>
+      <c r="G161" s="45" t="inlineStr">
+        <is>
+          <t>6.08</t>
+        </is>
+      </c>
+      <c r="H161" s="45" t="inlineStr">
+        <is>
+          <t>PO CO 3K (nie 5K): deload=mały koszt, ostatni czysty benchmark przed Teneryfą, test VO2/prędkości (5K już mamy), łatwiej trzymać RÓWNE tempo. Realny VDOT bez sandbaga. Pas piersiowy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B162" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C162" s="41" t="inlineStr">
+        <is>
+          <t>Easy 8 km</t>
+        </is>
+      </c>
+      <c r="D162" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E162" s="41" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F162" s="41" t="inlineStr"/>
+      <c r="G162" s="41" t="inlineStr">
+        <is>
+          <t>7.08</t>
+        </is>
+      </c>
+      <c r="H162" s="41" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="41" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B163" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C163" s="41" t="inlineStr">
+        <is>
+          <t>Recovery 6 km</t>
+        </is>
+      </c>
+      <c r="D163" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E163" s="41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F163" s="41" t="inlineStr"/>
+      <c r="G163" s="41" t="inlineStr">
+        <is>
+          <t>8.08</t>
+        </is>
+      </c>
+      <c r="H163" s="41" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="47" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B164" s="48" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="C164" s="47" t="inlineStr">
+        <is>
+          <t>Long 18 km easy</t>
+        </is>
+      </c>
+      <c r="D164" s="47" t="inlineStr">
+        <is>
+          <t>5:40–6:15</t>
+        </is>
+      </c>
+      <c r="E164" s="47" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="F164" s="47" t="inlineStr"/>
+      <c r="G164" s="47" t="inlineStr">
+        <is>
+          <t>9.08</t>
+        </is>
+      </c>
+      <c r="H164" s="47" t="inlineStr">
+        <is>
+          <t>po TT rekalibracja W17+</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="41" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B165" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C165" s="41" t="inlineStr">
+        <is>
+          <t>opcjonalnie rest zamiast easy</t>
+        </is>
+      </c>
+      <c r="D165" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E165" s="41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F165" s="41" t="inlineStr"/>
+      <c r="G165" s="41" t="inlineStr"/>
+      <c r="H165" s="41" t="inlineStr">
+        <is>
+          <t>deload = świeżość</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="49" t="n"/>
+      <c r="B166" s="49" t="n"/>
+      <c r="C166" s="49" t="n"/>
+      <c r="D166" s="50" t="inlineStr">
+        <is>
+          <t>SUMA km:</t>
+        </is>
+      </c>
+      <c r="E166" s="50" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="F166" s="49" t="n"/>
+      <c r="G166" s="49" t="n"/>
+      <c r="H166" s="50" t="inlineStr">
+        <is>
+          <t>Jeśli 3K &lt; 11:30 → VDOT 54+, akcenty −3–4 s/km.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="38" t="inlineStr">
+        <is>
+          <t>TYDZIEŃ 17 — 🏝️ TENERYFA tydz.1 / OBÓZ WYSOKOŚCIOWY (~83 km)</t>
+        </is>
+      </c>
+      <c r="B167" s="39" t="n"/>
+      <c r="C167" s="39" t="n"/>
+      <c r="D167" s="39" t="n"/>
+      <c r="E167" s="39" t="n"/>
+      <c r="F167" s="39" t="n"/>
+      <c r="G167" s="39" t="n"/>
+      <c r="H167" s="39" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="40" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B168" s="40" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="C168" s="40" t="inlineStr">
+        <is>
+          <t>Trening</t>
+        </is>
+      </c>
+      <c r="D168" s="40" t="inlineStr">
+        <is>
+          <t>Tempo /km</t>
+        </is>
+      </c>
+      <c r="E168" s="40" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="F168" s="40" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G168" s="40" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="H168" s="40" t="inlineStr">
+        <is>
+          <t>Notatki / feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B169" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C169" s="41" t="inlineStr">
+        <is>
+          <t>Przylot — shakeout 6 km (promenada) lub rest</t>
+        </is>
+      </c>
+      <c r="D169" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E169" s="41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F169" s="41" t="inlineStr"/>
+      <c r="G169" s="41" t="inlineStr">
+        <is>
+          <t>10.08</t>
+        </is>
+      </c>
+      <c r="H169" s="41" t="inlineStr">
+        <is>
+          <t>lot rano, w Puerto ~południe</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="41" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B170" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C170" s="41" t="inlineStr">
+        <is>
+          <t>Easy 12 km + 6×100 strides (promenada/Taoro)</t>
+        </is>
+      </c>
+      <c r="D170" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E170" s="41" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F170" s="41" t="inlineStr"/>
+      <c r="G170" s="41" t="inlineStr">
+        <is>
+          <t>11.08</t>
+        </is>
+      </c>
+      <c r="H170" s="41" t="inlineStr">
+        <is>
+          <t>odbiór aut 10:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B171" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C171" s="41" t="inlineStr">
+        <is>
+          <t>Easy 10 km (dzień Loro Parque)</t>
+        </is>
+      </c>
+      <c r="D171" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E171" s="41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F171" s="41" t="inlineStr"/>
+      <c r="G171" s="41" t="inlineStr">
+        <is>
+          <t>12.08</t>
+        </is>
+      </c>
+      <c r="H171" s="41" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="47" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B172" s="48" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="C172" s="47" t="inlineStr">
+        <is>
+          <t>⛰️ ALT LONG #1 Siete Cañadas ~2200 m (buty TRAIL!)</t>
+        </is>
+      </c>
+      <c r="D172" s="47" t="inlineStr">
+        <is>
+          <t>wg HR &lt;152 (~2:00-2:20)</t>
+        </is>
+      </c>
+      <c r="E172" s="47" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F172" s="47" t="inlineStr"/>
+      <c r="G172" s="47" t="inlineStr">
+        <is>
+          <t>13.08</t>
+        </is>
+      </c>
+      <c r="H172" s="47" t="inlineStr">
+        <is>
+          <t>świt, +La Orotava w drodze. Tempo −20-30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="41" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B173" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C173" s="41" t="inlineStr">
+        <is>
+          <t>Teide rodzinny — easy touch 8 km @2200 m (opc.) lub rest</t>
+        </is>
+      </c>
+      <c r="D173" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E173" s="41" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F173" s="41" t="inlineStr"/>
+      <c r="G173" s="41" t="inlineStr">
+        <is>
+          <t>14.08</t>
+        </is>
+      </c>
+      <c r="H173" s="41" t="inlineStr">
+        <is>
+          <t>nogi lekkie na dzień górski</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B174" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C174" s="41" t="inlineStr">
+        <is>
+          <t>Easy 12 km + strides (święto, lokalnie)</t>
+        </is>
+      </c>
+      <c r="D174" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E174" s="41" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F174" s="41" t="inlineStr"/>
+      <c r="G174" s="41" t="inlineStr">
+        <is>
+          <t>15.08</t>
+        </is>
+      </c>
+      <c r="H174" s="41" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="41" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B175" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C175" s="41" t="inlineStr">
+        <is>
+          <t>Easy 10 km o świcie (dzień Garachico)</t>
+        </is>
+      </c>
+      <c r="D175" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E175" s="41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F175" s="41" t="inlineStr"/>
+      <c r="G175" s="41" t="inlineStr">
+        <is>
+          <t>16.08</t>
+        </is>
+      </c>
+      <c r="H175" s="41" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="49" t="n"/>
+      <c r="B176" s="49" t="n"/>
+      <c r="C176" s="49" t="n"/>
+      <c r="D176" s="50" t="inlineStr">
+        <is>
+          <t>SUMA km:</t>
+        </is>
+      </c>
+      <c r="E176" s="50" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="F176" s="49" t="n"/>
+      <c r="G176" s="49" t="n"/>
+      <c r="H176" s="50" t="inlineStr">
+        <is>
+          <t>Longi wg CZASU nie km. Intensywność = na dole.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="38" t="inlineStr">
+        <is>
+          <t>TYDZIEŃ 18 — 🏝️ TENERYFA tydz.2 / LONG #2 + HM-pace na dole (~82 km)</t>
+        </is>
+      </c>
+      <c r="B177" s="39" t="n"/>
+      <c r="C177" s="39" t="n"/>
+      <c r="D177" s="39" t="n"/>
+      <c r="E177" s="39" t="n"/>
+      <c r="F177" s="39" t="n"/>
+      <c r="G177" s="39" t="n"/>
+      <c r="H177" s="39" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="40" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B178" s="40" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="C178" s="40" t="inlineStr">
+        <is>
+          <t>Trening</t>
+        </is>
+      </c>
+      <c r="D178" s="40" t="inlineStr">
+        <is>
+          <t>Tempo /km</t>
+        </is>
+      </c>
+      <c r="E178" s="40" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="F178" s="40" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G178" s="40" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="H178" s="40" t="inlineStr">
+        <is>
+          <t>Notatki / feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B179" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C179" s="41" t="inlineStr">
+        <is>
+          <t>Easy 10 km + strides (dzień Las Teresitas)</t>
+        </is>
+      </c>
+      <c r="D179" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E179" s="41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F179" s="41" t="inlineStr"/>
+      <c r="G179" s="41" t="inlineStr">
+        <is>
+          <t>17.08</t>
+        </is>
+      </c>
+      <c r="H179" s="41" t="inlineStr">
+        <is>
+          <t>świt</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="47" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B180" s="48" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="C180" s="47" t="inlineStr">
+        <is>
+          <t>⛰️ ALT LONG #2 Siete Cañadas ~2200 m (opc. finał Montaña Blanca ~2400)</t>
+        </is>
+      </c>
+      <c r="D180" s="47" t="inlineStr">
+        <is>
+          <t>wg HR (~2:00-2:20)</t>
+        </is>
+      </c>
+      <c r="E180" s="47" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F180" s="47" t="inlineStr"/>
+      <c r="G180" s="47" t="inlineStr">
+        <is>
+          <t>18.08</t>
+        </is>
+      </c>
+      <c r="H180" s="47" t="inlineStr">
+        <is>
+          <t>OSTATNI Teide (auto do 23). Trail!</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B181" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C181" s="41" t="inlineStr">
+        <is>
+          <t>Easy 8 km (Los Gigantes + rejs)</t>
+        </is>
+      </c>
+      <c r="D181" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E181" s="41" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F181" s="41" t="inlineStr"/>
+      <c r="G181" s="41" t="inlineStr">
+        <is>
+          <t>19.08</t>
+        </is>
+      </c>
+      <c r="H181" s="41" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B182" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C182" s="41" t="inlineStr">
+        <is>
+          <t>Easy 10 km (Siam Park)</t>
+        </is>
+      </c>
+      <c r="D182" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E182" s="41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F182" s="41" t="inlineStr"/>
+      <c r="G182" s="41" t="inlineStr">
+        <is>
+          <t>20.08</t>
+        </is>
+      </c>
+      <c r="H182" s="41" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="43" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B183" s="44" t="inlineStr">
+        <is>
+          <t>THRESHOLD</t>
+        </is>
+      </c>
+      <c r="C183" s="43" t="inlineStr">
+        <is>
+          <t>HM-PACE na DOLE: WU 3 + 8 km @ 4:12 + CD 2 (płaska promenada)</t>
+        </is>
+      </c>
+      <c r="D183" s="43" t="inlineStr">
+        <is>
+          <t>4:10–4:14</t>
+        </is>
+      </c>
+      <c r="E183" s="43" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F183" s="43" t="inlineStr"/>
+      <c r="G183" s="43" t="inlineStr">
+        <is>
+          <t>21.08</t>
+        </is>
+      </c>
+      <c r="H183" s="43" t="inlineStr">
+        <is>
+          <t>trzyma ostrość HM (Praski za 15 dni). Z tatą (jego MP≈4:12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B184" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C184" s="41" t="inlineStr">
+        <is>
+          <t>Easy 8 km (Masca/plaża)</t>
+        </is>
+      </c>
+      <c r="D184" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E184" s="41" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F184" s="41" t="inlineStr"/>
+      <c r="G184" s="41" t="inlineStr">
+        <is>
+          <t>22.08</t>
+        </is>
+      </c>
+      <c r="H184" s="41" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="41" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B185" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C185" s="41" t="inlineStr">
+        <is>
+          <t>Easy 8 km promenada (oddanie aut 10:00, pakowanie)</t>
+        </is>
+      </c>
+      <c r="D185" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E185" s="41" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F185" s="41" t="inlineStr"/>
+      <c r="G185" s="41" t="inlineStr">
+        <is>
+          <t>23.08</t>
+        </is>
+      </c>
+      <c r="H185" s="41" t="inlineStr">
+        <is>
+          <t>ostatni bieg</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="49" t="n"/>
+      <c r="B186" s="49" t="n"/>
+      <c r="C186" s="49" t="n"/>
+      <c r="D186" s="50" t="inlineStr">
+        <is>
+          <t>SUMA km:</t>
+        </is>
+      </c>
+      <c r="E186" s="50" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="F186" s="49" t="n"/>
+      <c r="G186" s="49" t="n"/>
+      <c r="H186" s="50" t="inlineStr">
+        <is>
+          <t>Powrót 24.08 → W19 sharpen, uwaga re-entry dip dzień 5-8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="38" t="inlineStr">
+        <is>
+          <t>TYDZIEŃ 19 — SHARPEN (24-30.08) · ~80 km</t>
+        </is>
+      </c>
+      <c r="B187" s="39" t="n"/>
+      <c r="C187" s="39" t="n"/>
+      <c r="D187" s="39" t="n"/>
+      <c r="E187" s="39" t="n"/>
+      <c r="F187" s="39" t="n"/>
+      <c r="G187" s="39" t="n"/>
+      <c r="H187" s="39" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="40" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B188" s="40" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="C188" s="40" t="inlineStr">
+        <is>
+          <t>Trening</t>
+        </is>
+      </c>
+      <c r="D188" s="40" t="inlineStr">
+        <is>
+          <t>Tempo /km</t>
+        </is>
+      </c>
+      <c r="E188" s="40" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="F188" s="40" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G188" s="40" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="H188" s="40" t="inlineStr">
+        <is>
+          <t>Notatki / feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B189" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C189" s="41" t="inlineStr">
+        <is>
+          <t>Easy 10 km + strides</t>
+        </is>
+      </c>
+      <c r="D189" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E189" s="41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F189" s="41" t="inlineStr"/>
+      <c r="G189" s="41" t="inlineStr">
+        <is>
+          <t>24.08</t>
+        </is>
+      </c>
+      <c r="H189" s="41" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B190" s="44" t="inlineStr">
+        <is>
+          <t>THRESHOLD</t>
+        </is>
+      </c>
+      <c r="C190" s="43" t="inlineStr">
+        <is>
+          <t>BROKEN HM: 4×3 km @ HM-pace 4:10–4:12 (400 jog), Adios Pro 4</t>
+        </is>
+      </c>
+      <c r="D190" s="43" t="inlineStr">
+        <is>
+          <t>4:10–4:12</t>
+        </is>
+      </c>
+      <c r="E190" s="43" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="F190" s="43" t="inlineStr"/>
+      <c r="G190" s="43" t="inlineStr">
+        <is>
+          <t>25.08</t>
+        </is>
+      </c>
+      <c r="H190" s="43" t="inlineStr">
+        <is>
+          <t>kluczowa sesja ostrości</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B191" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C191" s="41" t="inlineStr">
+        <is>
+          <t>Easy 10 km</t>
+        </is>
+      </c>
+      <c r="D191" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E191" s="41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F191" s="41" t="inlineStr"/>
+      <c r="G191" s="41" t="inlineStr">
+        <is>
+          <t>26.08</t>
+        </is>
+      </c>
+      <c r="H191" s="41" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="45" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B192" s="46" t="inlineStr">
+        <is>
+          <t>VO2max</t>
+        </is>
+      </c>
+      <c r="C192" s="45" t="inlineStr">
+        <is>
+          <t>3 WU → 5×800 @ 3:04 (400 jog) → 2 CD</t>
+        </is>
+      </c>
+      <c r="D192" s="45" t="inlineStr">
+        <is>
+          <t>3:02–3:06</t>
+        </is>
+      </c>
+      <c r="E192" s="45" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F192" s="45" t="inlineStr"/>
+      <c r="G192" s="45" t="inlineStr">
+        <is>
+          <t>27.08</t>
+        </is>
+      </c>
+      <c r="H192" s="45" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="41" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B193" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C193" s="41" t="inlineStr">
+        <is>
+          <t>Easy 8 km</t>
+        </is>
+      </c>
+      <c r="D193" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E193" s="41" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F193" s="41" t="inlineStr"/>
+      <c r="G193" s="41" t="inlineStr">
+        <is>
+          <t>28.08</t>
+        </is>
+      </c>
+      <c r="H193" s="41" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B194" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C194" s="41" t="inlineStr">
+        <is>
+          <t>Easy 6 km / rest</t>
+        </is>
+      </c>
+      <c r="D194" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E194" s="41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F194" s="41" t="inlineStr"/>
+      <c r="G194" s="41" t="inlineStr">
+        <is>
+          <t>29.08</t>
+        </is>
+      </c>
+      <c r="H194" s="41" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="47" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B195" s="48" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="C195" s="47" t="inlineStr">
+        <is>
+          <t>Long 20 km easy</t>
+        </is>
+      </c>
+      <c r="D195" s="47" t="inlineStr">
+        <is>
+          <t>5:40–6:15</t>
+        </is>
+      </c>
+      <c r="E195" s="47" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F195" s="47" t="inlineStr"/>
+      <c r="G195" s="47" t="inlineStr">
+        <is>
+          <t>30.08</t>
+        </is>
+      </c>
+      <c r="H195" s="47" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="49" t="n"/>
+      <c r="B196" s="49" t="n"/>
+      <c r="C196" s="49" t="n"/>
+      <c r="D196" s="50" t="inlineStr">
+        <is>
+          <t>SUMA km:</t>
+        </is>
+      </c>
+      <c r="E196" s="50" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="F196" s="49" t="n"/>
+      <c r="G196" s="49" t="n"/>
+      <c r="H196" s="50" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="38" t="inlineStr">
+        <is>
+          <t>TYDZIEŃ 20 — TAPER + WYŚCIG (31.08-5.09) · ~50 km 🏁 PRASKI</t>
+        </is>
+      </c>
+      <c r="B197" s="39" t="n"/>
+      <c r="C197" s="39" t="n"/>
+      <c r="D197" s="39" t="n"/>
+      <c r="E197" s="39" t="n"/>
+      <c r="F197" s="39" t="n"/>
+      <c r="G197" s="39" t="n"/>
+      <c r="H197" s="39" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="40" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B198" s="40" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="C198" s="40" t="inlineStr">
+        <is>
+          <t>Trening</t>
+        </is>
+      </c>
+      <c r="D198" s="40" t="inlineStr">
+        <is>
+          <t>Tempo /km</t>
+        </is>
+      </c>
+      <c r="E198" s="40" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="F198" s="40" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G198" s="40" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="H198" s="40" t="inlineStr">
+        <is>
+          <t>Notatki / feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B199" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C199" s="41" t="inlineStr">
+        <is>
+          <t>Easy 10 km</t>
+        </is>
+      </c>
+      <c r="D199" s="41" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E199" s="41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F199" s="41" t="inlineStr"/>
+      <c r="G199" s="41" t="inlineStr">
+        <is>
+          <t>31.08</t>
+        </is>
+      </c>
+      <c r="H199" s="41" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B200" s="44" t="inlineStr">
+        <is>
+          <t>THRESHOLD</t>
+        </is>
+      </c>
+      <c r="C200" s="43" t="inlineStr">
+        <is>
+          <t>PRIMER: 2 WU + 3×1 km @ 4:10 (400 jog) + CD</t>
+        </is>
+      </c>
+      <c r="D200" s="43" t="inlineStr">
+        <is>
+          <t>4:08–4:10</t>
+        </is>
+      </c>
+      <c r="E200" s="43" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F200" s="43" t="inlineStr"/>
+      <c r="G200" s="43" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="H200" s="43" t="inlineStr">
+        <is>
+          <t>wtorek — ostatni bodziec</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B201" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C201" s="41" t="inlineStr">
+        <is>
+          <t>Easy 8 km</t>
+        </is>
+      </c>
+      <c r="D201" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E201" s="41" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F201" s="41" t="inlineStr"/>
+      <c r="G201" s="41" t="inlineStr">
+        <is>
+          <t>2.09</t>
+        </is>
+      </c>
+      <c r="H201" s="41" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B202" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C202" s="41" t="inlineStr">
+        <is>
+          <t>Easy 6 km + 4×100 stride</t>
+        </is>
+      </c>
+      <c r="D202" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E202" s="41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F202" s="41" t="inlineStr"/>
+      <c r="G202" s="41" t="inlineStr">
+        <is>
+          <t>3.09</t>
+        </is>
+      </c>
+      <c r="H202" s="41" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="41" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B203" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C203" s="41" t="inlineStr">
+        <is>
+          <t>Rozbieganie 5 km (shakeout)</t>
+        </is>
+      </c>
+      <c r="D203" s="41" t="inlineStr">
+        <is>
+          <t>6:00–6:30</t>
+        </is>
+      </c>
+      <c r="E203" s="41" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F203" s="41" t="inlineStr"/>
+      <c r="G203" s="41" t="inlineStr">
+        <is>
+          <t>4.09</t>
+        </is>
+      </c>
+      <c r="H203" s="41" t="inlineStr">
+        <is>
+          <t>luz przed startem</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B204" s="42" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C204" s="41" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D204" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E204" s="41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F204" s="41" t="inlineStr"/>
+      <c r="G204" s="41" t="inlineStr"/>
+      <c r="H204" s="41" t="inlineStr">
+        <is>
+          <t>pełny odpoczynek</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="53" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B205" s="54" t="inlineStr">
+        <is>
+          <t>RACE</t>
+        </is>
+      </c>
+      <c r="C205" s="53" t="inlineStr">
+        <is>
+          <t>🏁 HM PRASKI — CEL sub-1:30 (wyjść 4:12/km!)</t>
+        </is>
+      </c>
+      <c r="D205" s="53" t="inlineStr">
+        <is>
+          <t>4:10–4:14</t>
+        </is>
+      </c>
+      <c r="E205" s="53" t="inlineStr">
+        <is>
+          <t>21,1</t>
+        </is>
+      </c>
+      <c r="F205" s="53" t="inlineStr"/>
+      <c r="G205" s="53" t="inlineStr">
+        <is>
+          <t>5.09</t>
+        </is>
+      </c>
+      <c r="H205" s="53" t="inlineStr">
+        <is>
+          <t>Adios Pro 4. Negatyw z 2. połowy jeśli czuje</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="49" t="n"/>
+      <c r="B206" s="49" t="n"/>
+      <c r="C206" s="49" t="n"/>
+      <c r="D206" s="50" t="inlineStr">
+        <is>
+          <t>SUMA km:</t>
+        </is>
+      </c>
+      <c r="E206" s="50" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F206" s="49" t="n"/>
+      <c r="G206" s="49" t="n"/>
+      <c r="H206" s="50" t="inlineStr">
+        <is>
+          <t>Race-day: NIE wychodź na 4:20 (lekcja z 5K).</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="33" t="inlineStr">
+        <is>
+          <t>★ W13–W20 rozpisane szczegółowo powyżej (recalib po 5K 19:49 → VDOT 52-53). Poniżej tylko SZKIC bloku Cracovia (W21–25).</t>
+        </is>
+      </c>
+      <c r="B215" s="33" t="inlineStr"/>
+      <c r="C215" s="34" t="inlineStr"/>
+      <c r="D215" s="33" t="inlineStr"/>
+      <c r="E215" s="33" t="inlineStr"/>
+      <c r="F215" s="33" t="inlineStr"/>
+      <c r="G215" s="33" t="inlineStr"/>
+      <c r="H215" s="34" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="28" t="inlineStr">
+        <is>
+          <t>■ BLOK 4: INTER-RACE → CRACOVIA (6.09-11.10)</t>
+        </is>
+      </c>
+      <c r="B216" s="28" t="inlineStr"/>
+      <c r="C216" s="29" t="inlineStr"/>
+      <c r="D216" s="28" t="inlineStr"/>
+      <c r="E216" s="28" t="inlineStr"/>
+      <c r="F216" s="28" t="inlineStr"/>
+      <c r="G216" s="28" t="inlineStr"/>
+      <c r="H216" s="29" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="9" t="inlineStr">
         <is>
           <t>TYDZIEŃ</t>
         </is>
       </c>
-      <c r="B129" s="9" t="inlineStr">
+      <c r="B217" s="9" t="inlineStr">
         <is>
           <t>DATY</t>
         </is>
       </c>
-      <c r="C129" s="10" t="inlineStr">
+      <c r="C217" s="10" t="inlineStr">
         <is>
           <t>FAZA</t>
         </is>
       </c>
-      <c r="D129" s="9" t="inlineStr">
+      <c r="D217" s="9" t="inlineStr">
         <is>
           <t>km</t>
         </is>
       </c>
-      <c r="E129" s="9" t="inlineStr">
+      <c r="E217" s="9" t="inlineStr">
         <is>
           <t>KLUCZOWE SESJE</t>
         </is>
       </c>
-      <c r="F129" s="9" t="inlineStr"/>
-      <c r="G129" s="9" t="inlineStr"/>
-      <c r="H129" s="10" t="inlineStr"/>
-    </row>
-    <row r="130">
-      <c r="A130" s="35" t="inlineStr">
-        <is>
-          <t>W13</t>
-        </is>
-      </c>
-      <c r="B130" s="5" t="inlineStr">
-        <is>
-          <t>13-19.07</t>
-        </is>
-      </c>
-      <c r="C130" s="6" t="inlineStr">
-        <is>
-          <t>HM-spec</t>
-        </is>
-      </c>
-      <c r="D130" s="5" t="inlineStr">
-        <is>
-          <t>92</t>
-        </is>
-      </c>
-      <c r="E130" s="5" t="inlineStr">
-        <is>
-          <t>Próg 2×4 km @4:10 · VO2 5×1000 @3:52 · Long 24 z 8 km @HM-pace · easy reszta</t>
-        </is>
-      </c>
-      <c r="F130" s="5" t="inlineStr"/>
-      <c r="G130" s="5" t="inlineStr"/>
-      <c r="H130" s="6" t="inlineStr"/>
-    </row>
-    <row r="131">
-      <c r="A131" s="35" t="inlineStr">
-        <is>
-          <t>W14</t>
-        </is>
-      </c>
-      <c r="B131" s="5" t="inlineStr">
-        <is>
-          <t>20-26.07</t>
-        </is>
-      </c>
-      <c r="C131" s="6" t="inlineStr">
-        <is>
-          <t>HM-spec</t>
-        </is>
-      </c>
-      <c r="D131" s="5" t="inlineStr">
-        <is>
-          <t>95</t>
-        </is>
-      </c>
-      <c r="E131" s="5" t="inlineStr">
-        <is>
-          <t>Próg ciągły 6 km @4:12 · Toughness 6×1km @5K (200jog) · Long 26 z 10 km @HM · podbiegi</t>
-        </is>
-      </c>
-      <c r="F131" s="5" t="inlineStr"/>
-      <c r="G131" s="5" t="inlineStr"/>
-      <c r="H131" s="6" t="inlineStr"/>
-    </row>
-    <row r="132">
-      <c r="A132" s="35" t="inlineStr">
-        <is>
-          <t>W15</t>
-        </is>
-      </c>
-      <c r="B132" s="5" t="inlineStr">
-        <is>
-          <t>27.07-2.08</t>
-        </is>
-      </c>
-      <c r="C132" s="6" t="inlineStr">
-        <is>
-          <t>HM-spec</t>
-        </is>
-      </c>
-      <c r="D132" s="5" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="E132" s="5" t="inlineStr">
-        <is>
-          <t>Próg 2×5 km @4:10 · VO2 8×800 @3:50 · Long 24 z 12 km @HM-pace</t>
-        </is>
-      </c>
-      <c r="F132" s="5" t="inlineStr"/>
-      <c r="G132" s="5" t="inlineStr"/>
-      <c r="H132" s="6" t="inlineStr"/>
-    </row>
-    <row r="133">
-      <c r="A133" s="35" t="inlineStr">
-        <is>
-          <t>W16</t>
-        </is>
-      </c>
-      <c r="B133" s="5" t="inlineStr">
-        <is>
-          <t>3-9.08</t>
-        </is>
-      </c>
-      <c r="C133" s="6" t="inlineStr">
-        <is>
-          <t>DELOAD + CHECK</t>
-        </is>
-      </c>
-      <c r="D133" s="5" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
-      <c r="E133" s="5" t="inlineStr">
-        <is>
-          <t>3K TT (sprawdzian VDOT) · easy · Long 18 — recalibracja tempa po TT</t>
-        </is>
-      </c>
-      <c r="F133" s="5" t="inlineStr"/>
-      <c r="G133" s="5" t="inlineStr"/>
-      <c r="H133" s="6" t="inlineStr"/>
-    </row>
-    <row r="134">
-      <c r="A134" s="5" t="inlineStr"/>
-      <c r="B134" s="5" t="inlineStr"/>
-      <c r="C134" s="6" t="inlineStr"/>
-      <c r="D134" s="5" t="inlineStr"/>
-      <c r="E134" s="5" t="inlineStr"/>
-      <c r="F134" s="5" t="inlineStr"/>
-      <c r="G134" s="5" t="inlineStr"/>
-      <c r="H134" s="6" t="inlineStr"/>
-    </row>
-    <row r="135">
-      <c r="A135" s="28" t="inlineStr">
-        <is>
-          <t>■ BLOK 3: HM PEAK + SHARPEN → PRASKI (10.08-5.09)</t>
-        </is>
-      </c>
-      <c r="B135" s="28" t="inlineStr"/>
-      <c r="C135" s="29" t="inlineStr"/>
-      <c r="D135" s="28" t="inlineStr"/>
-      <c r="E135" s="28" t="inlineStr"/>
-      <c r="F135" s="28" t="inlineStr"/>
-      <c r="G135" s="28" t="inlineStr"/>
-      <c r="H135" s="29" t="inlineStr"/>
-    </row>
-    <row r="136">
-      <c r="A136" s="9" t="inlineStr">
-        <is>
-          <t>TYDZIEŃ</t>
-        </is>
-      </c>
-      <c r="B136" s="9" t="inlineStr">
-        <is>
-          <t>DATY</t>
-        </is>
-      </c>
-      <c r="C136" s="10" t="inlineStr">
-        <is>
-          <t>FAZA</t>
-        </is>
-      </c>
-      <c r="D136" s="9" t="inlineStr">
-        <is>
-          <t>km</t>
-        </is>
-      </c>
-      <c r="E136" s="9" t="inlineStr">
-        <is>
-          <t>KLUCZOWE SESJE</t>
-        </is>
-      </c>
-      <c r="F136" s="9" t="inlineStr"/>
-      <c r="G136" s="9" t="inlineStr"/>
-      <c r="H136" s="10" t="inlineStr"/>
-    </row>
-    <row r="137">
-      <c r="A137" s="35" t="inlineStr">
-        <is>
-          <t>W17</t>
-        </is>
-      </c>
-      <c r="B137" s="5" t="inlineStr">
-        <is>
-          <t>10-16.08</t>
-        </is>
-      </c>
-      <c r="C137" s="6" t="inlineStr">
-        <is>
-          <t>PEAK</t>
-        </is>
-      </c>
-      <c r="D137" s="5" t="inlineStr">
-        <is>
-          <t>95</t>
-        </is>
-      </c>
-      <c r="E137" s="5" t="inlineStr">
-        <is>
-          <t>Próg 2×5 km @4:08 · Long 28 z 14 km @HM-pace · VO2 podtrzymanie</t>
-        </is>
-      </c>
-      <c r="F137" s="5" t="inlineStr"/>
-      <c r="G137" s="5" t="inlineStr"/>
-      <c r="H137" s="6" t="inlineStr"/>
-    </row>
-    <row r="138">
-      <c r="A138" s="35" t="inlineStr">
-        <is>
-          <t>W18</t>
-        </is>
-      </c>
-      <c r="B138" s="5" t="inlineStr">
-        <is>
-          <t>17-23.08</t>
-        </is>
-      </c>
-      <c r="C138" s="6" t="inlineStr">
-        <is>
-          <t>PEAK</t>
-        </is>
-      </c>
-      <c r="D138" s="5" t="inlineStr">
-        <is>
-          <t>96</t>
-        </is>
-      </c>
-      <c r="E138" s="5" t="inlineStr">
-        <is>
-          <t>HM-pace 16 km ciągłe @4:30 (race sim) · Long 26 · reps na świeżość</t>
-        </is>
-      </c>
-      <c r="F138" s="5" t="inlineStr"/>
-      <c r="G138" s="5" t="inlineStr"/>
-      <c r="H138" s="6" t="inlineStr"/>
-    </row>
-    <row r="139">
-      <c r="A139" s="35" t="inlineStr">
-        <is>
-          <t>W19</t>
-        </is>
-      </c>
-      <c r="B139" s="5" t="inlineStr">
-        <is>
-          <t>24-30.08</t>
-        </is>
-      </c>
-      <c r="C139" s="6" t="inlineStr">
+      <c r="F217" s="9" t="inlineStr"/>
+      <c r="G217" s="9" t="inlineStr"/>
+      <c r="H217" s="10" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="35" t="inlineStr">
+        <is>
+          <t>W21</t>
+        </is>
+      </c>
+      <c r="B218" s="5" t="inlineStr">
+        <is>
+          <t>7-13.09</t>
+        </is>
+      </c>
+      <c r="C218" s="6" t="inlineStr">
+        <is>
+          <t>RECOVER</t>
+        </is>
+      </c>
+      <c r="D218" s="5" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E218" s="5" t="inlineStr">
+        <is>
+          <t>3-4 dni easy/regen · jeden lekki próg pod koniec tyg · Long 16</t>
+        </is>
+      </c>
+      <c r="F218" s="5" t="inlineStr"/>
+      <c r="G218" s="5" t="inlineStr"/>
+      <c r="H218" s="6" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="35" t="inlineStr">
+        <is>
+          <t>W22</t>
+        </is>
+      </c>
+      <c r="B219" s="5" t="inlineStr">
+        <is>
+          <t>14-20.09</t>
+        </is>
+      </c>
+      <c r="C219" s="6" t="inlineStr">
+        <is>
+          <t>RE-SHARPEN</t>
+        </is>
+      </c>
+      <c r="D219" s="5" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="E219" s="5" t="inlineStr">
+        <is>
+          <t>Próg 2×4 km @4:08 · Long 24 z 10 km @HM · VO2 6×1000</t>
+        </is>
+      </c>
+      <c r="F219" s="5" t="inlineStr"/>
+      <c r="G219" s="5" t="inlineStr"/>
+      <c r="H219" s="6" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="35" t="inlineStr">
+        <is>
+          <t>W23</t>
+        </is>
+      </c>
+      <c r="B220" s="5" t="inlineStr">
+        <is>
+          <t>21-27.09</t>
+        </is>
+      </c>
+      <c r="C220" s="6" t="inlineStr">
+        <is>
+          <t>RE-SHARPEN</t>
+        </is>
+      </c>
+      <c r="D220" s="5" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="E220" s="5" t="inlineStr">
+        <is>
+          <t>HM-pace 12 km ciągłe · Long 22 · reps</t>
+        </is>
+      </c>
+      <c r="F220" s="5" t="inlineStr"/>
+      <c r="G220" s="5" t="inlineStr"/>
+      <c r="H220" s="6" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="35" t="inlineStr">
+        <is>
+          <t>W24</t>
+        </is>
+      </c>
+      <c r="B221" s="5" t="inlineStr">
+        <is>
+          <t>28.09-4.10</t>
+        </is>
+      </c>
+      <c r="C221" s="6" t="inlineStr">
         <is>
           <t>SHARPEN</t>
         </is>
       </c>
-      <c r="D139" s="5" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="E139" s="5" t="inlineStr">
-        <is>
-          <t>Broken HM: 4×3 km @HM-pace (400 jog) w Adios Pro 4 · short VO2 · Long 20</t>
-        </is>
-      </c>
-      <c r="F139" s="5" t="inlineStr"/>
-      <c r="G139" s="5" t="inlineStr"/>
-      <c r="H139" s="6" t="inlineStr"/>
-    </row>
-    <row r="140">
-      <c r="A140" s="35" t="inlineStr">
-        <is>
-          <t>W20</t>
-        </is>
-      </c>
-      <c r="B140" s="5" t="inlineStr">
-        <is>
-          <t>31.08-5.09</t>
-        </is>
-      </c>
-      <c r="C140" s="6" t="inlineStr">
+      <c r="D221" s="5" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E221" s="5" t="inlineStr">
+        <is>
+          <t>Broken HM 3×3 km @HM (Adios Pro 4) · easy · Long 18</t>
+        </is>
+      </c>
+      <c r="F221" s="5" t="inlineStr"/>
+      <c r="G221" s="5" t="inlineStr"/>
+      <c r="H221" s="6" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="35" t="inlineStr">
+        <is>
+          <t>W25</t>
+        </is>
+      </c>
+      <c r="B222" s="5" t="inlineStr">
+        <is>
+          <t>5-11.10</t>
+        </is>
+      </c>
+      <c r="C222" s="6" t="inlineStr">
         <is>
           <t>TAPER + RACE</t>
         </is>
       </c>
-      <c r="D140" s="5" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
-      <c r="E140" s="5" t="inlineStr">
-        <is>
-          <t>Easy + 2 WU+3×1km @4:10 (wt) · 5.09 HM PRASKI sub-1:35 (noc 20:30, Adios Pro 4)</t>
-        </is>
-      </c>
-      <c r="F140" s="5" t="inlineStr"/>
-      <c r="G140" s="5" t="inlineStr"/>
-      <c r="H140" s="6" t="inlineStr"/>
-    </row>
-    <row r="141">
-      <c r="A141" s="5" t="inlineStr"/>
-      <c r="B141" s="5" t="inlineStr"/>
-      <c r="C141" s="6" t="inlineStr"/>
-      <c r="D141" s="5" t="inlineStr"/>
-      <c r="E141" s="5" t="inlineStr"/>
-      <c r="F141" s="5" t="inlineStr"/>
-      <c r="G141" s="5" t="inlineStr"/>
-      <c r="H141" s="6" t="inlineStr"/>
-    </row>
-    <row r="142">
-      <c r="A142" s="28" t="inlineStr">
-        <is>
-          <t>■ BLOK 4: INTER-RACE → CRACOVIA (6.09-11.10)</t>
-        </is>
-      </c>
-      <c r="B142" s="28" t="inlineStr"/>
-      <c r="C142" s="29" t="inlineStr"/>
-      <c r="D142" s="28" t="inlineStr"/>
-      <c r="E142" s="28" t="inlineStr"/>
-      <c r="F142" s="28" t="inlineStr"/>
-      <c r="G142" s="28" t="inlineStr"/>
-      <c r="H142" s="29" t="inlineStr"/>
-    </row>
-    <row r="143">
-      <c r="A143" s="9" t="inlineStr">
-        <is>
-          <t>TYDZIEŃ</t>
-        </is>
-      </c>
-      <c r="B143" s="9" t="inlineStr">
-        <is>
-          <t>DATY</t>
-        </is>
-      </c>
-      <c r="C143" s="10" t="inlineStr">
-        <is>
-          <t>FAZA</t>
-        </is>
-      </c>
-      <c r="D143" s="9" t="inlineStr">
-        <is>
-          <t>km</t>
-        </is>
-      </c>
-      <c r="E143" s="9" t="inlineStr">
-        <is>
-          <t>KLUCZOWE SESJE</t>
-        </is>
-      </c>
-      <c r="F143" s="9" t="inlineStr"/>
-      <c r="G143" s="9" t="inlineStr"/>
-      <c r="H143" s="10" t="inlineStr"/>
-    </row>
-    <row r="144">
-      <c r="A144" s="35" t="inlineStr">
-        <is>
-          <t>W21</t>
-        </is>
-      </c>
-      <c r="B144" s="5" t="inlineStr">
-        <is>
-          <t>7-13.09</t>
-        </is>
-      </c>
-      <c r="C144" s="6" t="inlineStr">
-        <is>
-          <t>RECOVER</t>
-        </is>
-      </c>
-      <c r="D144" s="5" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="E144" s="5" t="inlineStr">
-        <is>
-          <t>3-4 dni easy/regen · jeden lekki próg pod koniec tyg · Long 16</t>
-        </is>
-      </c>
-      <c r="F144" s="5" t="inlineStr"/>
-      <c r="G144" s="5" t="inlineStr"/>
-      <c r="H144" s="6" t="inlineStr"/>
-    </row>
-    <row r="145">
-      <c r="A145" s="35" t="inlineStr">
-        <is>
-          <t>W22</t>
-        </is>
-      </c>
-      <c r="B145" s="5" t="inlineStr">
-        <is>
-          <t>14-20.09</t>
-        </is>
-      </c>
-      <c r="C145" s="6" t="inlineStr">
-        <is>
-          <t>RE-SHARPEN</t>
-        </is>
-      </c>
-      <c r="D145" s="5" t="inlineStr">
-        <is>
-          <t>86</t>
-        </is>
-      </c>
-      <c r="E145" s="5" t="inlineStr">
-        <is>
-          <t>Próg 2×4 km @4:08 · Long 24 z 10 km @HM · VO2 6×1000</t>
-        </is>
-      </c>
-      <c r="F145" s="5" t="inlineStr"/>
-      <c r="G145" s="5" t="inlineStr"/>
-      <c r="H145" s="6" t="inlineStr"/>
-    </row>
-    <row r="146">
-      <c r="A146" s="35" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B146" s="5" t="inlineStr">
-        <is>
-          <t>21-27.09</t>
-        </is>
-      </c>
-      <c r="C146" s="6" t="inlineStr">
-        <is>
-          <t>RE-SHARPEN</t>
-        </is>
-      </c>
-      <c r="D146" s="5" t="inlineStr">
-        <is>
-          <t>82</t>
-        </is>
-      </c>
-      <c r="E146" s="5" t="inlineStr">
-        <is>
-          <t>HM-pace 12 km ciągłe · Long 22 · reps</t>
-        </is>
-      </c>
-      <c r="F146" s="5" t="inlineStr"/>
-      <c r="G146" s="5" t="inlineStr"/>
-      <c r="H146" s="6" t="inlineStr"/>
-    </row>
-    <row r="147">
-      <c r="A147" s="35" t="inlineStr">
-        <is>
-          <t>W24</t>
-        </is>
-      </c>
-      <c r="B147" s="5" t="inlineStr">
-        <is>
-          <t>28.09-4.10</t>
-        </is>
-      </c>
-      <c r="C147" s="6" t="inlineStr">
-        <is>
-          <t>SHARPEN</t>
-        </is>
-      </c>
-      <c r="D147" s="5" t="inlineStr">
-        <is>
-          <t>66</t>
-        </is>
-      </c>
-      <c r="E147" s="5" t="inlineStr">
-        <is>
-          <t>Broken HM 3×3 km @HM (Adios Pro 4) · easy · Long 18</t>
-        </is>
-      </c>
-      <c r="F147" s="5" t="inlineStr"/>
-      <c r="G147" s="5" t="inlineStr"/>
-      <c r="H147" s="6" t="inlineStr"/>
-    </row>
-    <row r="148">
-      <c r="A148" s="35" t="inlineStr">
-        <is>
-          <t>W25</t>
-        </is>
-      </c>
-      <c r="B148" s="5" t="inlineStr">
-        <is>
-          <t>5-11.10</t>
-        </is>
-      </c>
-      <c r="C148" s="6" t="inlineStr">
-        <is>
-          <t>TAPER + RACE</t>
-        </is>
-      </c>
-      <c r="D148" s="5" t="inlineStr">
+      <c r="D222" s="5" t="inlineStr">
         <is>
           <t>46</t>
         </is>
       </c>
-      <c r="E148" s="5" t="inlineStr">
+      <c r="E222" s="5" t="inlineStr">
         <is>
           <t>Easy + krótki primer (wt 4×400 @4:00) · 11.10 CRACOVIA sub-1:33 PB</t>
         </is>
       </c>
-      <c r="F148" s="5" t="inlineStr"/>
-      <c r="G148" s="5" t="inlineStr"/>
-      <c r="H148" s="6" t="inlineStr"/>
-    </row>
-    <row r="149">
-      <c r="A149" s="5" t="inlineStr"/>
-      <c r="B149" s="5" t="inlineStr"/>
-      <c r="C149" s="6" t="inlineStr"/>
-      <c r="D149" s="5" t="inlineStr"/>
-      <c r="E149" s="5" t="inlineStr"/>
-      <c r="F149" s="5" t="inlineStr"/>
-      <c r="G149" s="5" t="inlineStr"/>
-      <c r="H149" s="6" t="inlineStr"/>
-    </row>
-    <row r="150">
-      <c r="A150" s="28" t="inlineStr">
+      <c r="F222" s="5" t="inlineStr"/>
+      <c r="G222" s="5" t="inlineStr"/>
+      <c r="H222" s="6" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="5" t="inlineStr"/>
+      <c r="B223" s="5" t="inlineStr"/>
+      <c r="C223" s="6" t="inlineStr"/>
+      <c r="D223" s="5" t="inlineStr"/>
+      <c r="E223" s="5" t="inlineStr"/>
+      <c r="F223" s="5" t="inlineStr"/>
+      <c r="G223" s="5" t="inlineStr"/>
+      <c r="H223" s="6" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="28" t="inlineStr">
         <is>
           <t>■ ZASADY</t>
         </is>
       </c>
-      <c r="B150" s="28" t="inlineStr"/>
-      <c r="C150" s="29" t="inlineStr"/>
-      <c r="D150" s="28" t="inlineStr"/>
-      <c r="E150" s="28" t="inlineStr"/>
-      <c r="F150" s="28" t="inlineStr"/>
-      <c r="G150" s="28" t="inlineStr"/>
-      <c r="H150" s="29" t="inlineStr"/>
-    </row>
-    <row r="151">
-      <c r="A151" s="5" t="inlineStr">
+      <c r="B224" s="28" t="inlineStr"/>
+      <c r="C224" s="29" t="inlineStr"/>
+      <c r="D224" s="28" t="inlineStr"/>
+      <c r="E224" s="28" t="inlineStr"/>
+      <c r="F224" s="28" t="inlineStr"/>
+      <c r="G224" s="28" t="inlineStr"/>
+      <c r="H224" s="29" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="5" t="inlineStr">
         <is>
           <t>1. Próg = PRAWDZIWY próg teraz (4:08-4:13, HR ~170+), nie Z3 4:30. To główny unlock.</t>
         </is>
       </c>
-      <c r="B151" s="5" t="inlineStr"/>
-      <c r="C151" s="6" t="inlineStr"/>
-      <c r="D151" s="5" t="inlineStr"/>
-      <c r="E151" s="5" t="inlineStr"/>
-      <c r="F151" s="5" t="inlineStr"/>
-      <c r="G151" s="5" t="inlineStr"/>
-      <c r="H151" s="6" t="inlineStr"/>
-    </row>
-    <row r="152">
-      <c r="A152" s="5" t="inlineStr">
+      <c r="B225" s="5" t="inlineStr"/>
+      <c r="C225" s="6" t="inlineStr"/>
+      <c r="D225" s="5" t="inlineStr"/>
+      <c r="E225" s="5" t="inlineStr"/>
+      <c r="F225" s="5" t="inlineStr"/>
+      <c r="G225" s="5" t="inlineStr"/>
+      <c r="H225" s="6" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="5" t="inlineStr">
         <is>
           <t>2. Toughness/race-pace reps z KRÓTKĄ przerwą — celowo niewygodne, bo limiter to głowa (patrz 5K finish 3:45 = miał zapas).</t>
         </is>
       </c>
-      <c r="B152" s="5" t="inlineStr"/>
-      <c r="C152" s="6" t="inlineStr"/>
-      <c r="D152" s="5" t="inlineStr"/>
-      <c r="E152" s="5" t="inlineStr"/>
-      <c r="F152" s="5" t="inlineStr"/>
-      <c r="G152" s="5" t="inlineStr"/>
-      <c r="H152" s="6" t="inlineStr"/>
-    </row>
-    <row r="153">
-      <c r="A153" s="5" t="inlineStr">
+      <c r="B226" s="5" t="inlineStr"/>
+      <c r="C226" s="6" t="inlineStr"/>
+      <c r="D226" s="5" t="inlineStr"/>
+      <c r="E226" s="5" t="inlineStr"/>
+      <c r="F226" s="5" t="inlineStr"/>
+      <c r="G226" s="5" t="inlineStr"/>
+      <c r="H226" s="6" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="5" t="inlineStr">
         <is>
           <t>3. 80/20: ~80% objętości EASY naprawdę wolno. Quality 2×/tydz + long. Mimo 8h snu — deload co 4 tyg święty.</t>
         </is>
       </c>
-      <c r="B153" s="5" t="inlineStr"/>
-      <c r="C153" s="6" t="inlineStr"/>
-      <c r="D153" s="5" t="inlineStr"/>
-      <c r="E153" s="5" t="inlineStr"/>
-      <c r="F153" s="5" t="inlineStr"/>
-      <c r="G153" s="5" t="inlineStr"/>
-      <c r="H153" s="6" t="inlineStr"/>
-    </row>
-    <row r="154">
-      <c r="A154" s="5" t="inlineStr">
-        <is>
-          <t>4. Pacing HM: pierwsza połowa 4:30-4:32, druga 4:28 — negatywny split. Trenuj to na longach (fast finish).</t>
-        </is>
-      </c>
-      <c r="B154" s="5" t="inlineStr"/>
-      <c r="C154" s="6" t="inlineStr"/>
-      <c r="D154" s="5" t="inlineStr"/>
-      <c r="E154" s="5" t="inlineStr"/>
-      <c r="F154" s="5" t="inlineStr"/>
-      <c r="G154" s="5" t="inlineStr"/>
-      <c r="H154" s="6" t="inlineStr"/>
-    </row>
-    <row r="155">
-      <c r="A155" s="5" t="inlineStr">
+      <c r="B227" s="5" t="inlineStr"/>
+      <c r="C227" s="6" t="inlineStr"/>
+      <c r="D227" s="5" t="inlineStr"/>
+      <c r="E227" s="5" t="inlineStr"/>
+      <c r="F227" s="5" t="inlineStr"/>
+      <c r="G227" s="5" t="inlineStr"/>
+      <c r="H227" s="6" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="5" t="inlineStr">
+        <is>
+          <t>4. Pacing HM (recalib): trzymaj 4:12/km od startu, negatyw z 2. połowy jeśli czuje. NIE wychodź na 4:20 (sandbag jak 5K 12.07).</t>
+        </is>
+      </c>
+      <c r="B228" s="5" t="inlineStr"/>
+      <c r="C228" s="6" t="inlineStr"/>
+      <c r="D228" s="5" t="inlineStr"/>
+      <c r="E228" s="5" t="inlineStr"/>
+      <c r="F228" s="5" t="inlineStr"/>
+      <c r="G228" s="5" t="inlineStr"/>
+      <c r="H228" s="6" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="5" t="inlineStr">
         <is>
           <t>5. Adios Pro 4: kup teraz, dotrzyj 2-3× HM-pace przed Praskim. Easy/long w trenażerach.</t>
         </is>
       </c>
-      <c r="B155" s="5" t="inlineStr"/>
-      <c r="C155" s="6" t="inlineStr"/>
-      <c r="D155" s="5" t="inlineStr"/>
-      <c r="E155" s="5" t="inlineStr"/>
-      <c r="F155" s="5" t="inlineStr"/>
-      <c r="G155" s="5" t="inlineStr"/>
-      <c r="H155" s="6" t="inlineStr"/>
-    </row>
-    <row r="156">
-      <c r="A156" s="5" t="inlineStr">
+      <c r="B229" s="5" t="inlineStr"/>
+      <c r="C229" s="6" t="inlineStr"/>
+      <c r="D229" s="5" t="inlineStr"/>
+      <c r="E229" s="5" t="inlineStr"/>
+      <c r="F229" s="5" t="inlineStr"/>
+      <c r="G229" s="5" t="inlineStr"/>
+      <c r="H229" s="6" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="5" t="inlineStr">
         <is>
           <t>6. Maciek nagminnie robi +5-15% nad plan — to OK przy jego regeneracji, ale w deloadach trzymaj plan.</t>
         </is>
       </c>
-      <c r="B156" s="5" t="inlineStr"/>
-      <c r="C156" s="6" t="inlineStr"/>
-      <c r="D156" s="5" t="inlineStr"/>
-      <c r="E156" s="5" t="inlineStr"/>
-      <c r="F156" s="5" t="inlineStr"/>
-      <c r="G156" s="5" t="inlineStr"/>
-      <c r="H156" s="6" t="inlineStr"/>
+      <c r="B230" s="5" t="inlineStr"/>
+      <c r="C230" s="6" t="inlineStr"/>
+      <c r="D230" s="5" t="inlineStr"/>
+      <c r="E230" s="5" t="inlineStr"/>
+      <c r="F230" s="5" t="inlineStr"/>
+      <c r="G230" s="5" t="inlineStr"/>
+      <c r="H230" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
coaching: uzasadnienie per jednostka W13-W16 Maciek (Notatki) + why-3K
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/maciek_plan_full.xlsx
+++ b/data/maciek_plan_full.xlsx
@@ -4590,7 +4590,7 @@
       </c>
       <c r="H129" s="41" t="inlineStr">
         <is>
-          <t>luźno, nogi po teście</t>
+          <t>→ zejście po 5K TT — świeżość na jakość · luźno, nogi po teście</t>
         </is>
       </c>
     </row>
@@ -4626,7 +4626,11 @@
           <t>14.07</t>
         </is>
       </c>
-      <c r="H130" s="41" t="inlineStr"/>
+      <c r="H130" s="41" t="inlineStr">
+        <is>
+          <t>→ objętość Z2 + strides = otwarcie neuromuskularne bez kosztu</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="43" t="inlineStr">
@@ -4662,7 +4666,7 @@
       </c>
       <c r="H131" s="43" t="inlineStr">
         <is>
-          <t>NA TEMPIE od 1. odcinka</t>
+          <t>→ GŁÓWNY akcent tyg — wytrzymałość progowa, baza pod HM-pace · NA TEMPIE od 1. odcinka</t>
         </is>
       </c>
     </row>
@@ -4698,7 +4702,11 @@
           <t>16.07</t>
         </is>
       </c>
-      <c r="H132" s="41" t="inlineStr"/>
+      <c r="H132" s="41" t="inlineStr">
+        <is>
+          <t>→ aeroba między jakościami</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="45" t="inlineStr">
@@ -4734,7 +4742,7 @@
       </c>
       <c r="H133" s="45" t="inlineStr">
         <is>
-          <t>pas piersiowy na HR</t>
+          <t>→ VO2/top-end — pułap nad progiem · pas piersiowy na HR</t>
         </is>
       </c>
     </row>
@@ -4770,7 +4778,11 @@
           <t>19.07</t>
         </is>
       </c>
-      <c r="H134" s="41" t="inlineStr"/>
+      <c r="H134" s="41" t="inlineStr">
+        <is>
+          <t>→ czyszczenie nóg przed longiem</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="47" t="inlineStr">
@@ -4806,7 +4818,7 @@
       </c>
       <c r="H135" s="47" t="inlineStr">
         <is>
-          <t>long spływa na pon</t>
+          <t>→ wytrzymałość + końcówka HM-pace = specyfika wyścigu · long spływa na pon</t>
         </is>
       </c>
     </row>
@@ -4920,7 +4932,11 @@
           <t>20.07</t>
         </is>
       </c>
-      <c r="H139" s="41" t="inlineStr"/>
+      <c r="H139" s="41" t="inlineStr">
+        <is>
+          <t>→ baza Z2</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="43" t="inlineStr">
@@ -4956,7 +4972,7 @@
       </c>
       <c r="H140" s="43" t="inlineStr">
         <is>
-          <t>trening trzymania tempa</t>
+          <t>→ trening TRZYMANIA tempa (Twój pacing) — bez przerw</t>
         </is>
       </c>
     </row>
@@ -4992,7 +5008,11 @@
           <t>22.07</t>
         </is>
       </c>
-      <c r="H141" s="41" t="inlineStr"/>
+      <c r="H141" s="41" t="inlineStr">
+        <is>
+          <t>→ regeneracja aerobowa</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="51" t="inlineStr">
@@ -5028,7 +5048,7 @@
       </c>
       <c r="H142" s="51" t="inlineStr">
         <is>
-          <t>limiter — tolerancja wys. HR</t>
+          <t>→ tolerancja wysokiego HR = Twój limiter (krótka przerwa celowo) · limiter — tolerancja wys. HR</t>
         </is>
       </c>
     </row>
@@ -5064,7 +5084,11 @@
           <t>24.07</t>
         </is>
       </c>
-      <c r="H143" s="41" t="inlineStr"/>
+      <c r="H143" s="41" t="inlineStr">
+        <is>
+          <t>→ luz</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="51" t="inlineStr">
@@ -5098,7 +5122,11 @@
           <t>25.07</t>
         </is>
       </c>
-      <c r="H144" s="51" t="inlineStr"/>
+      <c r="H144" s="51" t="inlineStr">
+        <is>
+          <t>→ siła biegowa + ekonomia, zero kosztu tempowego</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="47" t="inlineStr">
@@ -5134,7 +5162,7 @@
       </c>
       <c r="H145" s="47" t="inlineStr">
         <is>
-          <t>cap longa 26–28</t>
+          <t>→ największy long + duża dawka HM-pace · cap longa 26–28</t>
         </is>
       </c>
     </row>
@@ -5244,7 +5272,11 @@
           <t>27.07</t>
         </is>
       </c>
-      <c r="H149" s="41" t="inlineStr"/>
+      <c r="H149" s="41" t="inlineStr">
+        <is>
+          <t>→ baza Z2</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="43" t="inlineStr">
@@ -5280,7 +5312,7 @@
       </c>
       <c r="H150" s="43" t="inlineStr">
         <is>
-          <t>tempo od startu odcinka</t>
+          <t>→ dłuższe progi — wytrzymałość progowa rośnie · tempo od startu odcinka</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5348,11 @@
           <t>29.07</t>
         </is>
       </c>
-      <c r="H151" s="41" t="inlineStr"/>
+      <c r="H151" s="41" t="inlineStr">
+        <is>
+          <t>→ regeneracja aerobowa</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="45" t="inlineStr">
@@ -5350,7 +5386,11 @@
           <t>30.07</t>
         </is>
       </c>
-      <c r="H152" s="45" t="inlineStr"/>
+      <c r="H152" s="45" t="inlineStr">
+        <is>
+          <t>→ VO2/prędkość — ostrość</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="41" t="inlineStr">
@@ -5384,7 +5424,11 @@
           <t>31.07</t>
         </is>
       </c>
-      <c r="H153" s="41" t="inlineStr"/>
+      <c r="H153" s="41" t="inlineStr">
+        <is>
+          <t>→ luz</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="41" t="inlineStr">
@@ -5420,7 +5464,7 @@
       </c>
       <c r="H154" s="41" t="inlineStr">
         <is>
-          <t>sobota luz</t>
+          <t>→ świeżość przed longiem · sobota luz</t>
         </is>
       </c>
     </row>
@@ -5458,7 +5502,7 @@
       </c>
       <c r="H155" s="47" t="inlineStr">
         <is>
-          <t>najdłuższy blok race-pace</t>
+          <t>→ najdłuższy blok race-pace przed deloadem</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5616,11 @@
           <t>3.08</t>
         </is>
       </c>
-      <c r="H159" s="41" t="inlineStr"/>
+      <c r="H159" s="41" t="inlineStr">
+        <is>
+          <t>→ deload — schodzimy ze zmęczenia</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="41" t="inlineStr">
@@ -5608,7 +5656,7 @@
       </c>
       <c r="H160" s="41" t="inlineStr">
         <is>
-          <t>primer przed TT</t>
+          <t>→ primer przed TT — otwarcie nóg · primer przed TT</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5730,11 @@
           <t>7.08</t>
         </is>
       </c>
-      <c r="H162" s="41" t="inlineStr"/>
+      <c r="H162" s="41" t="inlineStr">
+        <is>
+          <t>→ regeneracja po TT</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="41" t="inlineStr">
@@ -5716,7 +5768,11 @@
           <t>8.08</t>
         </is>
       </c>
-      <c r="H163" s="41" t="inlineStr"/>
+      <c r="H163" s="41" t="inlineStr">
+        <is>
+          <t>→ luz przed longiem</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="47" t="inlineStr">
@@ -5752,7 +5808,7 @@
       </c>
       <c r="H164" s="47" t="inlineStr">
         <is>
-          <t>po TT rekalibracja W17+</t>
+          <t>→ aeroba + po TT recalibracja tempa · po TT rekalibracja W17+</t>
         </is>
       </c>
     </row>
@@ -7120,6 +7176,14 @@
         </is>
       </c>
     </row>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
     <row r="215">
       <c r="A215" s="33" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: 800m repy — '@ 3:04' czytane jako tempo/km (kosmos); jasno 3:48-3:52/km (≈3:04/800)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/maciek_plan_full.xlsx
+++ b/data/maciek_plan_full.xlsx
@@ -5367,12 +5367,12 @@
       </c>
       <c r="C152" s="45" t="inlineStr">
         <is>
-          <t>3 WU → 8×800 @ 3:04 (400 jog) → 2 CD</t>
+          <t>3 WU → 8×800 @ 3:48-3:52/km (≈3:04/800) (400 jog) → 2 CD</t>
         </is>
       </c>
       <c r="D152" s="45" t="inlineStr">
         <is>
-          <t>3:02–3:06</t>
+          <t>3:48-3:52/km</t>
         </is>
       </c>
       <c r="E152" s="45" t="inlineStr">
@@ -6707,12 +6707,12 @@
       </c>
       <c r="C192" s="45" t="inlineStr">
         <is>
-          <t>3 WU → 5×800 @ 3:04 (400 jog) → 2 CD</t>
+          <t>3 WU → 5×800 @ 3:48-3:52/km (≈3:04/800) (400 jog) → 2 CD</t>
         </is>
       </c>
       <c r="D192" s="45" t="inlineStr">
         <is>
-          <t>3:02–3:06</t>
+          <t>3:48-3:52/km</t>
         </is>
       </c>
       <c r="E192" s="45" t="inlineStr">

</xml_diff>

<commit_message>
fix: 'czyszczenie nóg' → rozluźnienie po VO2 (W13 sob)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/maciek_plan_full.xlsx
+++ b/data/maciek_plan_full.xlsx
@@ -4780,7 +4780,7 @@
       </c>
       <c r="H134" s="41" t="inlineStr">
         <is>
-          <t>→ czyszczenie nóg przed longiem</t>
+          <t>→ rozluźnienie po VO2, luźne nogi na niedzielny long</t>
         </is>
       </c>
     </row>
@@ -7176,14 +7176,6 @@
         </is>
       </c>
     </row>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
     <row r="215">
       <c r="A215" s="33" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: W13 kolizja 20.07 (long+easy) — long na nd 19.07, VO2/recovery cofnięte o dzień
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/maciek_plan_full.xlsx
+++ b/data/maciek_plan_full.xlsx
@@ -4737,7 +4737,7 @@
       <c r="F133" s="45" t="inlineStr"/>
       <c r="G133" s="45" t="inlineStr">
         <is>
-          <t>18.07</t>
+          <t>17.07</t>
         </is>
       </c>
       <c r="H133" s="45" t="inlineStr">
@@ -4775,7 +4775,7 @@
       <c r="F134" s="41" t="inlineStr"/>
       <c r="G134" s="41" t="inlineStr">
         <is>
-          <t>19.07</t>
+          <t>18.07</t>
         </is>
       </c>
       <c r="H134" s="41" t="inlineStr">
@@ -4813,12 +4813,12 @@
       <c r="F135" s="47" t="inlineStr"/>
       <c r="G135" s="47" t="inlineStr">
         <is>
-          <t>20.07</t>
+          <t>19.07</t>
         </is>
       </c>
       <c r="H135" s="47" t="inlineStr">
         <is>
-          <t>→ wytrzymałość + końcówka HM-pace = specyfika wyścigu · long spływa na pon</t>
+          <t>→ wytrzymałość + końcówka HM-pace = specyfika wyścigu</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: kolizja 13.07 (W12 regen = W13 pon) — W12 domyka się na teście 12.07
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/maciek_plan_full.xlsx
+++ b/data/maciek_plan_full.xlsx
@@ -4447,7 +4447,7 @@
       </c>
       <c r="C124" s="13" t="inlineStr">
         <is>
-          <t>Easy regen po teście (opc.)</t>
+          <t>Easy regen po teście → ujęte w W13 (pon 13.07)</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
@@ -4461,12 +4461,12 @@
         </is>
       </c>
       <c r="F124" s="11" t="inlineStr"/>
-      <c r="G124" s="11" t="inlineStr">
-        <is>
-          <t>13.07</t>
-        </is>
-      </c>
-      <c r="H124" s="13" t="inlineStr"/>
+      <c r="G124" s="11" t="inlineStr"/>
+      <c r="H124" s="13" t="inlineStr">
+        <is>
+          <t>nie liczyć podwójnie — recovery 13.07 jest w W13</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="17" t="inlineStr"/>

</xml_diff>

<commit_message>
10.08 (przylot) = REST bez biegu; km rozłożone na inne dni (Maciek W17 + Tomasz T14)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/maciek_plan_full.xlsx
+++ b/data/maciek_plan_full.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -170,8 +170,13 @@
       <color rgb="00AD1457"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00607D8B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -243,6 +248,11 @@
         <fgColor rgb="00FDE7EF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECEFF1"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -284,7 +294,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -414,6 +424,8 @@
     <xf numFmtId="0" fontId="25" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5925,40 +5937,40 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="41" t="inlineStr">
+      <c r="A169" s="55" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B169" s="42" t="inlineStr">
-        <is>
-          <t>EASY</t>
-        </is>
-      </c>
-      <c r="C169" s="41" t="inlineStr">
-        <is>
-          <t>Przylot — shakeout 6 km (promenada) lub rest</t>
-        </is>
-      </c>
-      <c r="D169" s="41" t="inlineStr">
-        <is>
-          <t>6:00–6:30</t>
-        </is>
-      </c>
-      <c r="E169" s="41" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="F169" s="41" t="inlineStr"/>
-      <c r="G169" s="41" t="inlineStr">
+      <c r="B169" s="56" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="C169" s="55" t="inlineStr">
+        <is>
+          <t>Przylot — BEZ biegu (dojazd z TFS, zameldowanie La Paz)</t>
+        </is>
+      </c>
+      <c r="D169" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E169" s="55" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F169" s="55" t="inlineStr"/>
+      <c r="G169" s="55" t="inlineStr">
         <is>
           <t>10.08</t>
         </is>
       </c>
-      <c r="H169" s="41" t="inlineStr">
-        <is>
-          <t>lot rano, w Puerto ~południe</t>
+      <c r="H169" s="55" t="inlineStr">
+        <is>
+          <t>nie da rady po podróży — dzień wolny</t>
         </is>
       </c>
     </row>
@@ -5975,7 +5987,7 @@
       </c>
       <c r="C170" s="41" t="inlineStr">
         <is>
-          <t>Easy 12 km + 6×100 strides (promenada/Taoro)</t>
+          <t>Easy 14 km + 6×100 m strides (promenada/Taoro)</t>
         </is>
       </c>
       <c r="D170" s="41" t="inlineStr">
@@ -5985,7 +5997,7 @@
       </c>
       <c r="E170" s="41" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>14</t>
         </is>
       </c>
       <c r="F170" s="41" t="inlineStr"/>
@@ -6013,7 +6025,7 @@
       </c>
       <c r="C171" s="41" t="inlineStr">
         <is>
-          <t>Easy 10 km (dzień Loro Parque)</t>
+          <t>Easy 12 km (dzień Loro Parque)</t>
         </is>
       </c>
       <c r="D171" s="41" t="inlineStr">
@@ -6023,7 +6035,7 @@
       </c>
       <c r="E171" s="41" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F171" s="41" t="inlineStr"/>
@@ -6157,7 +6169,7 @@
       </c>
       <c r="C175" s="41" t="inlineStr">
         <is>
-          <t>Easy 10 km o świcie (dzień Garachico)</t>
+          <t>Easy 12 km o świcie (dzień Garachico)</t>
         </is>
       </c>
       <c r="D175" s="41" t="inlineStr">
@@ -6167,7 +6179,7 @@
       </c>
       <c r="E175" s="41" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F175" s="41" t="inlineStr"/>
@@ -6196,7 +6208,7 @@
       <c r="G176" s="49" t="n"/>
       <c r="H176" s="50" t="inlineStr">
         <is>
-          <t>Longi wg CZASU nie km. Intensywność = na dole.</t>
+          <t>km z 10.08 (przylot) rozłożone na 11/12/16.08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
maciek Praski: strategia negatyw start ~4:15 (grupa 1:30 jeśli będzie / zegarek), uspójniona z lekcją 5K
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/maciek_plan_full.xlsx
+++ b/data/maciek_plan_full.xlsx
@@ -7141,7 +7141,7 @@
       </c>
       <c r="C205" s="53" t="inlineStr">
         <is>
-          <t>🏁 HM PRASKI — CEL sub-1:30 (wyjść 4:12/km!)</t>
+          <t>🏁 HM PRASKI (nocny 20:30) — CEL sub-1:30 (realnie 1:28-1:29)</t>
         </is>
       </c>
       <c r="D205" s="53" t="inlineStr">
@@ -7162,7 +7162,7 @@
       </c>
       <c r="H205" s="53" t="inlineStr">
         <is>
-          <t>Adios Pro 4. Negatyw z 2. połowy jeśli czuje</t>
+          <t>NEGATYW: km 0-5 @ ~4:15 (grupa 1:30 jeśli wystartuje, inaczej wg zegarka) → km 5-16 @ 4:10-4:12 → km 16-21 @ 4:05-4:08. Adios Pro 4.</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
     <row r="228">
       <c r="A228" s="5" t="inlineStr">
         <is>
-          <t>4. Pacing HM (recalib): trzymaj 4:12/km od startu, negatyw z 2. połowy jeśli czuje. NIE wychodź na 4:20 (sandbag jak 5K 12.07).</t>
+          <t>4. Pacing HM = NEGATYW: start ~4:15 przez 3-5 km (grupa 1:30 jeśli będzie / wg zegarka — kontrola, NIE wolniej niż 4:16), potem 4:10-4:12, finisz 4:05-4:08 → 1:27-1:29. NIE zostawaj na 4:15 dłużej niż 5 km.</t>
         </is>
       </c>
       <c r="B228" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
maciek Praski: usuń '4:12 od startu', negatyw z grupą 1:30 (~4:15) jako plan bazowy
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/maciek_plan_full.xlsx
+++ b/data/maciek_plan_full.xlsx
@@ -7162,7 +7162,7 @@
       </c>
       <c r="H205" s="53" t="inlineStr">
         <is>
-          <t>NEGATYW: km 0-5 @ ~4:15 (grupa 1:30 jeśli wystartuje, inaczej wg zegarka) → km 5-16 @ 4:10-4:12 → km 16-21 @ 4:05-4:08. Adios Pro 4.</t>
+          <t>NEGATYW: km 0-5 z grupą 1:30 (~4:15) → km 5-16 @ 4:10-4:12 → km 16-21 @ 4:05-4:08. Adios Pro 4.</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
     <row r="228">
       <c r="A228" s="5" t="inlineStr">
         <is>
-          <t>4. Pacing HM = NEGATYW: start ~4:15 przez 3-5 km (grupa 1:30 jeśli będzie / wg zegarka — kontrola, NIE wolniej niż 4:16), potem 4:10-4:12, finisz 4:05-4:08 → 1:27-1:29. NIE zostawaj na 4:15 dłużej niż 5 km.</t>
+          <t>4. Pacing HM = NEGATYW: start ~4:15 z grupą 1:30 przez 3-5 km (kontrola, NIE wolniej niż 4:16), potem 4:10-4:12, finisz 4:05-4:08 → 1:27-1:29. NIE zostawaj z grupą 1:30 dłużej niż 5 km.</t>
         </is>
       </c>
       <c r="B228" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
maciek: spacing fix — 1 jakość mid-week (ŚRODA, 72h po longu) + long, nigdy 2 twarde w 48h
Lekcja 15-17.07: próg 2×4 + VO2 5×1000 @3:50 w 48h = zmęczony (planowe, nie przesadził).
Przy longu w niedzielę nie da się wcisnąć 2 jakości mid-week bez kolizji 48h → 1 jakość + long.
- W14: toughness usunięty, próg wt→śr (72h po longu). Podbiegi ≤10× wróciły jako neuromusk. (nie jakość).
- W15: VO2 8×800 usunięty, próg 2×5km wt→śr.
- W19: VO2 5×800 usunięty, broken HM pon→śr (re-entry z Teneryfy).
- ZASADY: mid-week jakość=środa; podbiegi/strides nie liczą się jako jakość; spacing to lever, nie cięcie km.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/maciek_plan_full.xlsx
+++ b/data/maciek_plan_full.xlsx
@@ -176,7 +176,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -253,6 +253,18 @@
         <fgColor rgb="00ECEFF1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E9F5E9"/>
+        <bgColor rgb="00E9F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBF3E0"/>
+        <bgColor rgb="00FBF3E0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -294,7 +306,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -426,6 +438,10 @@
     <xf numFmtId="0" fontId="26" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4951,116 +4967,110 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="43" t="inlineStr">
+      <c r="A140" s="57" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B140" s="44" t="inlineStr">
+      <c r="B140" s="58" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C140" s="57" t="inlineStr">
+        <is>
+          <t>Easy 10 km</t>
+        </is>
+      </c>
+      <c r="D140" s="57" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E140" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="F140" s="57" t="inlineStr"/>
+      <c r="G140" s="57" t="inlineStr">
+        <is>
+          <t>21.07</t>
+        </is>
+      </c>
+      <c r="H140" s="57" t="inlineStr">
+        <is>
+          <t>→ regen (48 h po niedzielnym longu — jakość dopiero śr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="59" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B141" s="60" t="inlineStr">
         <is>
           <t>THRESHOLD</t>
         </is>
       </c>
-      <c r="C140" s="43" t="inlineStr">
+      <c r="C141" s="59" t="inlineStr">
         <is>
           <t>PRÓG CIĄGŁY 6 km @ 4:12 (WU 3 + CD 3)</t>
         </is>
       </c>
-      <c r="D140" s="43" t="inlineStr">
+      <c r="D141" s="59" t="inlineStr">
         <is>
           <t>4:10–4:12</t>
         </is>
       </c>
-      <c r="E140" s="43" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="F140" s="43" t="inlineStr"/>
-      <c r="G140" s="43" t="inlineStr">
-        <is>
-          <t>21.07</t>
-        </is>
-      </c>
-      <c r="H140" s="43" t="inlineStr">
-        <is>
-          <t>→ trening TRZYMANIA tempa (Twój pacing) — bez przerw</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="41" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B141" s="42" t="inlineStr">
+      <c r="E141" s="59" t="n">
+        <v>12</v>
+      </c>
+      <c r="F141" s="59" t="inlineStr"/>
+      <c r="G141" s="59" t="inlineStr">
+        <is>
+          <t>22.07</t>
+        </is>
+      </c>
+      <c r="H141" s="59" t="inlineStr">
+        <is>
+          <t>→ jakość mid-week (śr = 72 h po longu) · trzymanie tempa bez przerw</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="57" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B142" s="58" t="inlineStr">
         <is>
           <t>EASY</t>
         </is>
       </c>
-      <c r="C141" s="41" t="inlineStr">
-        <is>
-          <t>Easy 10 km</t>
-        </is>
-      </c>
-      <c r="D141" s="41" t="inlineStr">
+      <c r="C142" s="57" t="inlineStr">
+        <is>
+          <t>Easy 8 km + 8× podbieg 40 s (trucht w dół)</t>
+        </is>
+      </c>
+      <c r="D142" s="57" t="inlineStr">
         <is>
           <t>5:50–6:30</t>
         </is>
       </c>
-      <c r="E141" s="41" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="F141" s="41" t="inlineStr"/>
-      <c r="G141" s="41" t="inlineStr">
-        <is>
-          <t>22.07</t>
-        </is>
-      </c>
-      <c r="H141" s="41" t="inlineStr">
-        <is>
-          <t>→ regeneracja aerobowa</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="51" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B142" s="52" t="inlineStr">
-        <is>
-          <t>TOUGHNESS</t>
-        </is>
-      </c>
-      <c r="C142" s="51" t="inlineStr">
-        <is>
-          <t>6×1000 @ 3:48–3:52, rec 200 m KRÓTKA (WU3+CD2)</t>
-        </is>
-      </c>
-      <c r="D142" s="51" t="inlineStr">
-        <is>
-          <t>3:48–3:52</t>
-        </is>
-      </c>
-      <c r="E142" s="51" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="F142" s="51" t="inlineStr"/>
-      <c r="G142" s="51" t="inlineStr">
+      <c r="E142" s="57" t="n">
+        <v>9</v>
+      </c>
+      <c r="F142" s="57" t="inlineStr"/>
+      <c r="G142" s="57" t="inlineStr">
         <is>
           <t>23.07</t>
         </is>
       </c>
-      <c r="H142" s="51" t="inlineStr">
-        <is>
-          <t>→ tolerancja wysokiego HR = Twój limiter (krótka przerwa celowo) · limiter — tolerancja wys. HR</t>
+      <c r="H142" s="57" t="inlineStr">
+        <is>
+          <t>→ podbiegi ≤10 = neuromuskularne, NIE jakość · siła/ekonomia bez kosztu tempowego</t>
         </is>
       </c>
     </row>
@@ -5103,40 +5113,38 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="51" t="inlineStr">
+      <c r="A144" s="57" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B144" s="52" t="inlineStr">
-        <is>
-          <t>HILL</t>
-        </is>
-      </c>
-      <c r="C144" s="51" t="inlineStr">
-        <is>
-          <t>Easy 6 + 8× podbieg 40 s + 2 CD</t>
-        </is>
-      </c>
-      <c r="D144" s="51" t="inlineStr">
-        <is>
-          <t>wysiłek</t>
-        </is>
-      </c>
-      <c r="E144" s="51" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="F144" s="51" t="inlineStr"/>
-      <c r="G144" s="51" t="inlineStr">
+      <c r="B144" s="58" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C144" s="57" t="inlineStr">
+        <is>
+          <t>Easy 9 km + 6×100 m stride</t>
+        </is>
+      </c>
+      <c r="D144" s="57" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E144" s="57" t="n">
+        <v>9</v>
+      </c>
+      <c r="F144" s="57" t="inlineStr"/>
+      <c r="G144" s="57" t="inlineStr">
         <is>
           <t>25.07</t>
         </is>
       </c>
-      <c r="H144" s="51" t="inlineStr">
-        <is>
-          <t>→ siła biegowa + ekonomia, zero kosztu tempowego</t>
+      <c r="H144" s="57" t="inlineStr">
+        <is>
+          <t>→ hill wycięty → 2 jakości/tydz (próg + toughness). Easy+strides tanio, świeże nogi na long 26 km</t>
         </is>
       </c>
     </row>
@@ -5291,116 +5299,110 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="43" t="inlineStr">
+      <c r="A150" s="57" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B150" s="44" t="inlineStr">
+      <c r="B150" s="58" t="inlineStr">
+        <is>
+          <t>EASY</t>
+        </is>
+      </c>
+      <c r="C150" s="57" t="inlineStr">
+        <is>
+          <t>Easy 12 km</t>
+        </is>
+      </c>
+      <c r="D150" s="57" t="inlineStr">
+        <is>
+          <t>5:50–6:30</t>
+        </is>
+      </c>
+      <c r="E150" s="57" t="n">
+        <v>12</v>
+      </c>
+      <c r="F150" s="57" t="inlineStr"/>
+      <c r="G150" s="57" t="inlineStr">
+        <is>
+          <t>28.07</t>
+        </is>
+      </c>
+      <c r="H150" s="57" t="inlineStr">
+        <is>
+          <t>→ regen (48 h po longu — jakość dopiero śr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="59" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B151" s="60" t="inlineStr">
         <is>
           <t>THRESHOLD</t>
         </is>
       </c>
-      <c r="C150" s="43" t="inlineStr">
+      <c r="C151" s="59" t="inlineStr">
         <is>
           <t>2 WU → 2×5 km @ 4:10 (800 jog) → 2 CD</t>
         </is>
       </c>
-      <c r="D150" s="43" t="inlineStr">
+      <c r="D151" s="59" t="inlineStr">
         <is>
           <t>4:08–4:12</t>
         </is>
       </c>
-      <c r="E150" s="43" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="F150" s="43" t="inlineStr"/>
-      <c r="G150" s="43" t="inlineStr">
-        <is>
-          <t>28.07</t>
-        </is>
-      </c>
-      <c r="H150" s="43" t="inlineStr">
-        <is>
-          <t>→ dłuższe progi — wytrzymałość progowa rośnie · tempo od startu odcinka</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="41" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B151" s="42" t="inlineStr">
+      <c r="E151" s="59" t="n">
+        <v>15</v>
+      </c>
+      <c r="F151" s="59" t="inlineStr"/>
+      <c r="G151" s="59" t="inlineStr">
+        <is>
+          <t>29.07</t>
+        </is>
+      </c>
+      <c r="H151" s="59" t="inlineStr">
+        <is>
+          <t>→ jakość mid-week (śr = 72 h po longu) · tempo od startu odcinka</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="57" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B152" s="58" t="inlineStr">
         <is>
           <t>EASY</t>
         </is>
       </c>
-      <c r="C151" s="41" t="inlineStr">
-        <is>
-          <t>Easy 12 km</t>
-        </is>
-      </c>
-      <c r="D151" s="41" t="inlineStr">
+      <c r="C152" s="57" t="inlineStr">
+        <is>
+          <t>Easy 10 km</t>
+        </is>
+      </c>
+      <c r="D152" s="57" t="inlineStr">
         <is>
           <t>5:50–6:30</t>
         </is>
       </c>
-      <c r="E151" s="41" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="F151" s="41" t="inlineStr"/>
-      <c r="G151" s="41" t="inlineStr">
-        <is>
-          <t>29.07</t>
-        </is>
-      </c>
-      <c r="H151" s="41" t="inlineStr">
-        <is>
-          <t>→ regeneracja aerobowa</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="45" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B152" s="46" t="inlineStr">
-        <is>
-          <t>VO2max</t>
-        </is>
-      </c>
-      <c r="C152" s="45" t="inlineStr">
-        <is>
-          <t>3 WU → 8×800 @ 3:48-3:52/km (≈3:04/800) (400 jog) → 2 CD</t>
-        </is>
-      </c>
-      <c r="D152" s="45" t="inlineStr">
-        <is>
-          <t>3:48-3:52/km</t>
-        </is>
-      </c>
-      <c r="E152" s="45" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="F152" s="45" t="inlineStr"/>
-      <c r="G152" s="45" t="inlineStr">
+      <c r="E152" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="F152" s="57" t="inlineStr"/>
+      <c r="G152" s="57" t="inlineStr">
         <is>
           <t>30.07</t>
         </is>
       </c>
-      <c r="H152" s="45" t="inlineStr">
-        <is>
-          <t>→ VO2/prędkość — ostrość</t>
+      <c r="H152" s="57" t="inlineStr">
+        <is>
+          <t>→ regen (VO2 usunięty — 1 jakość mid-week + long)</t>
         </is>
       </c>
     </row>
@@ -5417,7 +5419,7 @@
       </c>
       <c r="C153" s="41" t="inlineStr">
         <is>
-          <t>Easy 8 km</t>
+          <t>Easy 8 km + 8× podbieg 40 s (trucht w dół)</t>
         </is>
       </c>
       <c r="D153" s="41" t="inlineStr">
@@ -5425,10 +5427,8 @@
           <t>6:00–6:30</t>
         </is>
       </c>
-      <c r="E153" s="41" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="E153" s="41" t="n">
+        <v>9</v>
       </c>
       <c r="F153" s="41" t="inlineStr"/>
       <c r="G153" s="41" t="inlineStr">
@@ -5438,7 +5438,7 @@
       </c>
       <c r="H153" s="41" t="inlineStr">
         <is>
-          <t>→ luz</t>
+          <t>→ podbiegi ≤10 = neuromuskularne, NIE jakość · świeżość przed longiem OK</t>
         </is>
       </c>
     </row>
@@ -6601,38 +6601,40 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="41" t="inlineStr">
+      <c r="A189" s="57" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B189" s="42" t="inlineStr">
+      <c r="B189" s="58" t="inlineStr">
         <is>
           <t>EASY</t>
         </is>
       </c>
-      <c r="C189" s="41" t="inlineStr">
+      <c r="C189" s="57" t="inlineStr">
         <is>
           <t>Easy 10 km + strides</t>
         </is>
       </c>
-      <c r="D189" s="41" t="inlineStr">
+      <c r="D189" s="57" t="inlineStr">
         <is>
           <t>5:50–6:30</t>
         </is>
       </c>
-      <c r="E189" s="41" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="F189" s="41" t="inlineStr"/>
-      <c r="G189" s="41" t="inlineStr">
+      <c r="E189" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="F189" s="57" t="inlineStr"/>
+      <c r="G189" s="57" t="inlineStr">
         <is>
           <t>24.08</t>
         </is>
       </c>
-      <c r="H189" s="41" t="inlineStr"/>
+      <c r="H189" s="57" t="inlineStr">
+        <is>
+          <t>→ osiadanie po podróży/wysokości (broken HM przesunięty na śr)</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="43" t="inlineStr">
@@ -6673,38 +6675,40 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="41" t="inlineStr">
+      <c r="A191" s="59" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B191" s="42" t="inlineStr">
-        <is>
-          <t>EASY</t>
-        </is>
-      </c>
-      <c r="C191" s="41" t="inlineStr">
-        <is>
-          <t>Easy 10 km</t>
-        </is>
-      </c>
-      <c r="D191" s="41" t="inlineStr">
-        <is>
-          <t>5:50–6:30</t>
-        </is>
-      </c>
-      <c r="E191" s="41" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="F191" s="41" t="inlineStr"/>
-      <c r="G191" s="41" t="inlineStr">
+      <c r="B191" s="60" t="inlineStr">
+        <is>
+          <t>THRESHOLD</t>
+        </is>
+      </c>
+      <c r="C191" s="59" t="inlineStr">
+        <is>
+          <t>BROKEN HM: 4×3 km @ HM-pace 4:10–4:12 (400 jog), Adios Pro 4</t>
+        </is>
+      </c>
+      <c r="D191" s="59" t="inlineStr">
+        <is>
+          <t>4:10–4:12</t>
+        </is>
+      </c>
+      <c r="E191" s="59" t="n">
+        <v>18</v>
+      </c>
+      <c r="F191" s="59" t="inlineStr"/>
+      <c r="G191" s="59" t="inlineStr">
         <is>
           <t>26.08</t>
         </is>
       </c>
-      <c r="H191" s="41" t="inlineStr"/>
+      <c r="H191" s="59" t="inlineStr">
+        <is>
+          <t>→ kluczowy sharpener — 3 dni po powrocie, świeższe niż pon · realna specyfika (nogi po obozie)</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="45" t="inlineStr">
@@ -7299,7 +7303,7 @@
       </c>
       <c r="E219" s="5" t="inlineStr">
         <is>
-          <t>Próg 2×4 km @4:08 · Long 24 z 10 km @HM · VO2 6×1000</t>
+          <t>Próg 2×4 km @4:08 · Long 24 z 10 km @HM (1 jakość + long — spacing) · reps krótkie na świeżość</t>
         </is>
       </c>
       <c r="F219" s="5" t="inlineStr"/>
@@ -7451,7 +7455,7 @@
     <row r="227">
       <c r="A227" s="5" t="inlineStr">
         <is>
-          <t>3. 80/20: ~80% objętości EASY naprawdę wolno. Quality 2×/tydz + long. Mimo 8h snu — deload co 4 tyg święty.</t>
+          <t>3. 80/20 easy naprawdę wolno. HARD = 1 jakość mid-week + long z segmentem (2 twarde/tydz). Jakość mid-week = ŚRODA (72 h po niedzielnym longu; WTOREK = tylko 48 h po longu = za blisko). MIN 72 h między twardymi, NIGDY 2 w 48 h — lekcja 15-17.07: próg 2×4 + VO2 5×1000 @3:50 (planowe) w 48 h = zmęczony. Podbiegi ≤10× i strides = neuromuskularne, NIE jakość (mogą być na easy). Deload co 4 tyg święty.</t>
         </is>
       </c>
       <c r="B227" s="5" t="inlineStr"/>
@@ -7493,7 +7497,7 @@
     <row r="230">
       <c r="A230" s="5" t="inlineStr">
         <is>
-          <t>6. Maciek nagminnie robi +5-15% nad plan — to OK przy jego regeneracji, ale w deloadach trzymaj plan.</t>
+          <t>6. Maciek robi +5-15% km nad plan — to OK przy jego regeneracji. Zmęczenie 17.07 NIE z objętości, tylko z 2 twardych w 48 h — dlatego lever to SPACING, nie cięcie km. Jakość rób wg planu (nie dokładaj powtórzeń).</t>
         </is>
       </c>
       <c r="B230" s="5" t="inlineStr"/>

</xml_diff>